<commit_message>
daily auto-refresh 2026-09-14 15:01
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-21 11:40
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-22 13:00
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1091,10 +1091,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>bantzuk</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>akiatuconteh</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
@@ -1108,24 +1112,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-15 11:51:02</t>
+          <t>2026-09-09 07:32:58</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bantzuk</t>
+          <t>https://www.tiktok.com/@akiatuconteh</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>badmashi.007</t>
+          <t>a13dde</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1142,24 +1146,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-14 18:24:25</t>
+          <t>2026-09-14 08:25:14</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@badmashi.007</t>
+          <t>https://www.tiktok.com/@a13dde</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ali.syed873</t>
+          <t>atokeade053</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1176,24 +1180,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-17 03:47:33</t>
+          <t>2026-09-14 20:29:27</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ali.syed873</t>
+          <t>https://www.tiktok.com/@atokeade053</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>alemap9</t>
+          <t>anita.wils</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1210,24 +1214,24 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-14 00:26:00</t>
+          <t>2026-09-16 09:42:03</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@alemap9</t>
+          <t>https://www.tiktok.com/@anita.wils</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>a13dde</t>
+          <t>angelaugochinyere</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1244,35 +1248,31 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-14 08:25:14</t>
+          <t>2026-09-16 22:04:31</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@a13dde</t>
+          <t>https://www.tiktok.com/@angelaugochinyere</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>akiatuconteh</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
+          <t>allthingscutziee</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1282,24 +1282,24 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-09 07:32:58</t>
+          <t>2026-09-15 11:51:03</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@akiatuconteh</t>
+          <t>https://www.tiktok.com/@allthingscutziee</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>atokeade053</t>
+          <t>alemap9</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1316,24 +1316,24 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-14 20:29:27</t>
+          <t>2026-09-14 00:26:00</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@atokeade053</t>
+          <t>https://www.tiktok.com/@alemap9</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>anita.wils</t>
+          <t>ali.syed873</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:03</t>
+          <t>2026-09-17 03:47:33</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1360,14 +1360,14 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@anita.wils</t>
+          <t>https://www.tiktok.com/@ali.syed873</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>angelaugochinyere</t>
+          <t>barbaraasiedu771</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1384,31 +1384,31 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-16 22:04:31</t>
+          <t>2026-09-09 21:11:27</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@angelaugochinyere</t>
+          <t>https://www.tiktok.com/@barbaraasiedu771</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>allthingscutziee</t>
+          <t>badmashi.007</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1418,24 +1418,24 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-15 11:51:03</t>
+          <t>2026-09-14 18:24:25</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@allthingscutziee</t>
+          <t>https://www.tiktok.com/@badmashi.007</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>beauty20208</t>
+          <t>courageous527</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1452,24 +1452,24 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-18 19:31:55</t>
+          <t>2026-09-11 19:24:33</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@beauty20208</t>
+          <t>https://www.tiktok.com/@courageous527</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>barbaraasiedu771</t>
+          <t>dabrat1138</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-09 21:11:27</t>
+          <t>2026-09-10 01:03:04</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@barbaraasiedu771</t>
+          <t>https://www.tiktok.com/@dabrat1138</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1537,14 +1537,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>diane.docherty</t>
+          <t>dailymusthaves20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1554,92 +1554,92 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-15 09:50:59</t>
+          <t>2026-09-19 13:38:02</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@diane.docherty</t>
+          <t>https://www.tiktok.com/@dailymusthaves20</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>donsnewchapter</t>
+          <t>dollywithplaits73</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-16 09:45:02</t>
+          <t>2026-09-16 16:47:28</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@donsnewchapter</t>
+          <t>https://www.tiktok.com/@dollywithplaits73</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>dollywithplaits73</t>
+          <t>donsnewchapter</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-16 16:47:28</t>
+          <t>2026-09-16 09:45:02</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dollywithplaits73</t>
+          <t>https://www.tiktok.com/@donsnewchapter</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>dulal.miah2471</t>
+          <t>drantero_10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1656,24 +1656,24 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-14 07:26:09</t>
+          <t>2026-09-17 14:48:32</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dulal.miah2471</t>
+          <t>https://www.tiktok.com/@drantero_10</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>dy7yobwohcu6</t>
+          <t>diane.docherty</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1690,31 +1690,31 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-18 21:30:44</t>
+          <t>2026-09-15 09:50:59</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dy7yobwohcu6</t>
+          <t>https://www.tiktok.com/@diane.docherty</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>elizabethj27</t>
+          <t>bex_lifeafter40</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-10 23:49:16</t>
+          <t>2026-09-17 15:30:23</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@elizabethj27</t>
+          <t>https://www.tiktok.com/@bex_lifeafter40</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>drantero_10</t>
+          <t>bgee2345</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1758,17 +1758,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-17 14:48:32</t>
+          <t>2026-09-19 22:31:01</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@drantero_10</t>
+          <t>https://www.tiktok.com/@bgee2345</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1809,7 +1809,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>chucky692</t>
+          <t>bantzuk</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1826,85 +1826,85 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-15 07:29:48</t>
+          <t>2026-09-15 11:51:02</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chucky692</t>
+          <t>https://www.tiktok.com/@bantzuk</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>clairedipple66</t>
+          <t>beauty20208</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-16 07:44:02</t>
+          <t>2026-09-18 19:31:55</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@clairedipple66</t>
+          <t>https://www.tiktok.com/@beauty20208</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>be__beauty1</t>
+          <t>beemahempire</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-08 17:18:23</t>
+          <t>2026-09-15 11:52:03</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@be__beauty1</t>
+          <t>https://www.tiktok.com/@beemahempire</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -1945,75 +1945,75 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>bettyaddo398</t>
+          <t>be__beauty1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-14 14:52:28</t>
+          <t>2026-09-08 17:18:23</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bettyaddo398</t>
+          <t>https://www.tiktok.com/@be__beauty1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>bex_lifeafter40</t>
+          <t>gella4573</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-17 15:30:23</t>
+          <t>2026-09-16 07:50:13</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bex_lifeafter40</t>
+          <t>https://www.tiktok.com/@gella4573</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>beemahempire</t>
+          <t>fernandasprivy</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2030,31 +2030,31 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-15 11:52:03</t>
+          <t>2026-09-15 19:00:52</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@beemahempire</t>
+          <t>https://www.tiktok.com/@fernandasprivy</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>haseeb.mum</t>
+          <t>eni_folabi</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2064,126 +2064,126 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:03</t>
+          <t>2026-09-09 11:38:46</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@haseeb.mum</t>
+          <t>https://www.tiktok.com/@eni_folabi</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>gl80.31</t>
+          <t>emaanttshop</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-10 23:30:20</t>
+          <t>2026-09-15 21:32:02</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gl80.31</t>
+          <t>https://www.tiktok.com/@emaanttshop</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>georgiafergg</t>
+          <t>elizabethj27</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:03</t>
+          <t>2026-09-10 23:49:16</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@georgiafergg</t>
+          <t>https://www.tiktok.com/@elizabethj27</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>gella4573</t>
+          <t>hinas_beauty_buys</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-16 07:50:13</t>
+          <t>2026-09-18 09:46:05</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gella4573</t>
+          <t>https://www.tiktok.com/@hinas_beauty_buys</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fernandasprivy</t>
+          <t>hchahal80</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -2200,24 +2200,24 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-15 19:00:52</t>
+          <t>2026-09-15 20:35:21</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fernandasprivy</t>
+          <t>https://www.tiktok.com/@hchahal80</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>hrahmancookings</t>
+          <t>georgiafergg</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2234,17 +2234,17 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-08 19:45:29</t>
+          <t>2026-09-16 09:42:03</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hrahmancookings</t>
+          <t>https://www.tiktok.com/@georgiafergg</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2285,7 +2285,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>hchahal80</t>
+          <t>hrahmancookings</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
@@ -2302,31 +2302,31 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-15 20:35:21</t>
+          <t>2026-09-08 19:45:29</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hchahal80</t>
+          <t>https://www.tiktok.com/@hrahmancookings</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>is.colonel</t>
+          <t>iqrasumman19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-05 23:55:02</t>
+          <t>2026-09-19 22:51:02</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@is.colonel</t>
+          <t>https://www.tiktok.com/@iqrasumman19</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2455,14 +2455,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>jxnxxkxk</t>
+          <t>haseeb.mum</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-15 12:32:04</t>
+          <t>2026-09-16 09:42:03</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2482,14 +2482,14 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@jxnxxkxk</t>
+          <t>https://www.tiktok.com/@haseeb.mum</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>k.tee146</t>
+          <t>gl80.31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
@@ -2506,24 +2506,24 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-10 09:41:07</t>
+          <t>2026-09-10 23:30:20</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@k.tee146</t>
+          <t>https://www.tiktok.com/@gl80.31</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>iqrasumman19</t>
+          <t>k.tee146</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
@@ -2540,85 +2540,85 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-19 22:51:02</t>
+          <t>2026-09-10 09:41:07</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@iqrasumman19</t>
+          <t>https://www.tiktok.com/@k.tee146</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>hinas_beauty_buys</t>
+          <t>jxnxxkxk</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-18 09:46:05</t>
+          <t>2026-09-15 12:32:04</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hinas_beauty_buys</t>
+          <t>https://www.tiktok.com/@jxnxxkxk</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>kay.h0</t>
+          <t>kamo76710</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-09 04:27:35</t>
+          <t>2026-09-20 05:21:24</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kay.h0</t>
+          <t>https://www.tiktok.com/@kamo76710</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2659,14 +2659,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>kayyu247</t>
+          <t>keeskloset</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2676,31 +2676,31 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-09 09:42:51</t>
+          <t>2026-09-16 09:57:04</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kayyu247</t>
+          <t>https://www.tiktok.com/@keeskloset</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>keeskloset</t>
+          <t>kennybabe692</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2710,92 +2710,92 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-09-16 09:57:04</t>
+          <t>2026-09-10 11:43:02</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@keeskloset</t>
+          <t>https://www.tiktok.com/@kennybabe692</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>konaduroi</t>
+          <t>kay.h0</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-15 03:00:44</t>
+          <t>2026-09-09 04:27:35</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@konaduroi</t>
+          <t>https://www.tiktok.com/@kay.h0</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>lady_dash07</t>
+          <t>kayyu247</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-09-05 21:11:23</t>
+          <t>2026-09-09 09:42:51</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@lady_dash07</t>
+          <t>https://www.tiktok.com/@kayyu247</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>kennybabe692</t>
+          <t>dulal.miah2471</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
@@ -2812,24 +2812,24 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-10 11:43:02</t>
+          <t>2026-09-14 07:26:09</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kennybabe692</t>
+          <t>https://www.tiktok.com/@dulal.miah2471</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>kofoworola2853</t>
+          <t>dy7yobwohcu6</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
@@ -2846,17 +2846,17 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-11 10:52:59</t>
+          <t>2026-09-18 21:30:44</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kofoworola2853</t>
+          <t>https://www.tiktok.com/@dy7yobwohcu6</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -2897,68 +2897,68 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>emaanttshop</t>
+          <t>chucky692</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-15 21:32:02</t>
+          <t>2026-09-15 07:29:48</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@emaanttshop</t>
+          <t>https://www.tiktok.com/@chucky692</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>eni_folabi</t>
+          <t>clairedipple66</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-09 11:38:46</t>
+          <t>2026-09-16 07:44:02</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@eni_folabi</t>
+          <t>https://www.tiktok.com/@clairedipple66</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -2999,41 +2999,41 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>courageous527</t>
+          <t>claudia.claudia970</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-11 19:24:33</t>
+          <t>2026-09-20 22:09:26</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@courageous527</t>
+          <t>https://www.tiktok.com/@claudia.claudia970</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>dabrat1138</t>
+          <t>bettyaddo398</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
@@ -3050,31 +3050,31 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-09-10 01:03:04</t>
+          <t>2026-09-14 14:52:28</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dabrat1138</t>
+          <t>https://www.tiktok.com/@bettyaddo398</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>dailymusthaves20</t>
+          <t>missyspranno12</t>
         </is>
       </c>
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3084,24 +3084,24 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-09-19 13:38:02</t>
+          <t>2026-09-15 13:31:44</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dailymusthaves20</t>
+          <t>https://www.tiktok.com/@missyspranno12</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>bgee2345</t>
+          <t>mehmoonaali238</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
@@ -3118,92 +3118,92 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-09-19 22:31:01</t>
+          <t>2026-09-17 11:42:05</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bgee2345</t>
+          <t>https://www.tiktok.com/@mehmoonaali238</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>mlllifestyle</t>
+          <t>markh_8</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-18 09:46:03</t>
+          <t>2026-09-09 16:07:49</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mlllifestyle</t>
+          <t>https://www.tiktok.com/@markh_8</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>missyspranno12</t>
+          <t>maish1002</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-15 13:31:44</t>
+          <t>2026-09-19 13:31:02</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@missyspranno12</t>
+          <t>https://www.tiktok.com/@maish1002</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>mehmoonaali238</t>
+          <t>ladydonigbinosa</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
@@ -3220,126 +3220,126 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-09-17 11:42:05</t>
+          <t>2026-09-14 07:25:08</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mehmoonaali238</t>
+          <t>https://www.tiktok.com/@ladydonigbinosa</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>markh_8</t>
+          <t>lucia25070</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-09-09 16:07:49</t>
+          <t>2026-09-18 09:46:03</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@markh_8</t>
+          <t>https://www.tiktok.com/@lucia25070</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>lucia25070</t>
+          <t>kofoworola2853</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-09-18 09:46:03</t>
+          <t>2026-09-11 10:52:59</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@lucia25070</t>
+          <t>https://www.tiktok.com/@kofoworola2853</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>maish1002</t>
+          <t>konaduroi</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-09-19 13:31:02</t>
+          <t>2026-09-15 03:00:44</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@maish1002</t>
+          <t>https://www.tiktok.com/@konaduroi</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ladydonigbinosa</t>
+          <t>nrahi28</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
@@ -3356,41 +3356,41 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-14 07:25:08</t>
+          <t>2026-09-20 14:59:29</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ladydonigbinosa</t>
+          <t>https://www.tiktok.com/@nrahi28</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ladyygold1</t>
+          <t>oladayomartins</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-09-16 09:45:05</t>
+          <t>2026-09-17 21:17:16</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3400,7 +3400,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ladyygold1</t>
+          <t>https://www.tiktok.com/@oladayomartins</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3437,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3449,24 +3449,24 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>oluwatoyosiabayom</t>
+          <t>monicalavern</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-09-14 17:04:02</t>
+          <t>2026-09-15 13:00:13</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3476,14 +3476,14 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oluwatoyosiabayom</t>
+          <t>https://www.tiktok.com/@monicalavern</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>omolade.abebi</t>
+          <t>mz.jada0</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -3500,24 +3500,24 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-09-17 10:33:35</t>
+          <t>2026-09-07 21:15:37</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@omolade.abebi</t>
+          <t>https://www.tiktok.com/@mz.jada0</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>monicalavern</t>
+          <t>moon19867</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -3534,24 +3534,24 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-09-15 13:00:13</t>
+          <t>2026-09-11 19:21:54</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@monicalavern</t>
+          <t>https://www.tiktok.com/@moon19867</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>mz.jada0</t>
+          <t>muhammadsha110</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -3568,24 +3568,24 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-09-07 21:15:37</t>
+          <t>2026-09-11 15:36:47</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mz.jada0</t>
+          <t>https://www.tiktok.com/@muhammadsha110</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>moon19867</t>
+          <t>mymojomindset</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -3602,24 +3602,24 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-09-11 19:21:54</t>
+          <t>2026-09-15 10:29:05</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@moon19867</t>
+          <t>https://www.tiktok.com/@mymojomindset</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>muhammadsha110</t>
+          <t>padnerkupakuwana</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -3636,24 +3636,24 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-09-11 15:36:47</t>
+          <t>2026-09-13 02:02:06</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@muhammadsha110</t>
+          <t>https://www.tiktok.com/@padnerkupakuwana</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>mymojomindset</t>
+          <t>oyetunji.sunday</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -3670,31 +3670,31 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-09-15 10:29:05</t>
+          <t>2026-09-12 13:08:25</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mymojomindset</t>
+          <t>https://www.tiktok.com/@oyetunji.sunday</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>positiveproductsuk</t>
+          <t>ornellabeauty25</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -3704,17 +3704,17 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-09-15 11:53:04</t>
+          <t>2026-09-07 22:41:47</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@positiveproductsuk</t>
+          <t>https://www.tiktok.com/@ornellabeauty25</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -3755,7 +3755,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>padnerkupakuwana</t>
+          <t>r4xla15</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -3772,65 +3772,65 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-09-13 02:02:06</t>
+          <t>2026-09-20 15:22:42</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@padnerkupakuwana</t>
+          <t>https://www.tiktok.com/@r4xla15</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ranifarooq_3</t>
+          <t>queeen_0f_hearts</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-09-13 22:37:56</t>
+          <t>2026-09-13 23:51:38</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ranifarooq_3</t>
+          <t>https://www.tiktok.com/@queeen_0f_hearts</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>queeen_0f_hearts</t>
+          <t>positiveproductsuk</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -3840,31 +3840,31 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-09-13 23:51:38</t>
+          <t>2026-09-15 11:53:04</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@queeen_0f_hearts</t>
+          <t>https://www.tiktok.com/@positiveproductsuk</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>rory.the.cocker</t>
+          <t>ranifarooq_3</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -3874,58 +3874,58 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-09-18 18:13:02</t>
+          <t>2026-09-13 22:37:56</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rory.the.cocker</t>
+          <t>https://www.tiktok.com/@ranifarooq_3</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>rozana2026</t>
+          <t>rory.the.cocker</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-09-19 15:08:34</t>
+          <t>2026-09-18 18:13:02</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rozana2026</t>
+          <t>https://www.tiktok.com/@rory.the.cocker</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ruksi1607</t>
+          <t>rozana2026</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -3942,24 +3942,24 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-13 20:49:20</t>
+          <t>2026-09-19 15:08:34</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ruksi1607</t>
+          <t>https://www.tiktok.com/@rozana2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>saadia7166</t>
+          <t>ruksi1607</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -3976,58 +3976,58 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-09-10 11:16:51</t>
+          <t>2026-09-13 20:49:20</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@saadia7166</t>
+          <t>https://www.tiktok.com/@ruksi1607</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>sajarshed</t>
+          <t>oluwatoyosiabayom</t>
         </is>
       </c>
       <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-09-19 10:17:35</t>
+          <t>2026-09-14 17:04:02</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sajarshed</t>
+          <t>https://www.tiktok.com/@oluwatoyosiabayom</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>samirakarim24</t>
+          <t>omolade.abebi</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
@@ -4044,24 +4044,24 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-09-11 11:10:48</t>
+          <t>2026-09-17 10:33:35</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@samirakarim24</t>
+          <t>https://www.tiktok.com/@omolade.abebi</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ornellabeauty25</t>
+          <t>na2706_1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
@@ -4078,24 +4078,24 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-07 22:41:47</t>
+          <t>2026-09-20 23:38:18</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ornellabeauty25</t>
+          <t>https://www.tiktok.com/@na2706_1</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>oyetunji.sunday</t>
+          <t>nanahdaramy</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
@@ -4112,24 +4112,24 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-12 13:08:25</t>
+          <t>2026-09-14 00:12:20</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oyetunji.sunday</t>
+          <t>https://www.tiktok.com/@nanahdaramy</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>nanahdaramy</t>
+          <t>nancymm52</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -4146,31 +4146,31 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-14 00:12:20</t>
+          <t>2026-09-18 07:04:23</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nanahdaramy</t>
+          <t>https://www.tiktok.com/@nancymm52</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>nancymm52</t>
+          <t>sehrish2015</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4180,58 +4180,58 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-18 07:04:23</t>
+          <t>2026-09-16 09:42:03</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nancymm52</t>
+          <t>https://www.tiktok.com/@sehrish2015</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>oladayomartins</t>
+          <t>sedi546</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-17 21:17:16</t>
+          <t>2026-09-13 15:46:07</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oladayomartins</t>
+          <t>https://www.tiktok.com/@sedi546</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>shoni1984</t>
+          <t>samirakarim24</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -4248,7 +4248,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-10 08:20:01</t>
+          <t>2026-09-11 11:10:48</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -4258,21 +4258,21 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shoni1984</t>
+          <t>https://www.tiktok.com/@samirakarim24</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>shazzbegum0</t>
+          <t>sajarshed</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4282,24 +4282,24 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-15 11:58:02</t>
+          <t>2026-09-19 10:17:35</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shazzbegum0</t>
+          <t>https://www.tiktok.com/@sajarshed</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>sexybaby7657</t>
+          <t>saadia7166</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -4316,7 +4316,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-09 21:00:27</t>
+          <t>2026-09-10 11:16:51</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -4326,21 +4326,21 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sexybaby7657</t>
+          <t>https://www.tiktok.com/@saadia7166</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>sehrish2015</t>
+          <t>ste.baby6</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4350,24 +4350,24 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:03</t>
+          <t>2026-09-09 16:28:17</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sehrish2015</t>
+          <t>https://www.tiktok.com/@ste.baby6</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>sedi546</t>
+          <t>sjahan83</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -4384,58 +4384,58 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-09-13 15:46:07</t>
+          <t>2026-09-12 13:46:48</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sedi546</t>
+          <t>https://www.tiktok.com/@sjahan83</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>sweetshez1</t>
+          <t>sexybaby7657</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-09-05 18:50:17</t>
+          <t>2026-09-09 21:00:27</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sweetshez1</t>
+          <t>https://www.tiktok.com/@sexybaby7657</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ste.baby6</t>
+          <t>syrashid</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -4452,126 +4452,126 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-09-09 16:28:17</t>
+          <t>2026-09-11 12:35:39</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ste.baby6</t>
+          <t>https://www.tiktok.com/@syrashid</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>sjahan83</t>
+          <t>su.k806</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Shatavari 1300mg Extra Strength</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-12 13:46:48</t>
+          <t>2026-09-17 20:34:02</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sjahan83</t>
+          <t>https://www.tiktok.com/@su.k806</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>thehomelylondon</t>
+          <t>themamadee</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-18 15:51:23</t>
+          <t>2026-09-10 19:23:49</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@thehomelylondon</t>
+          <t>https://www.tiktok.com/@themamadee</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>theartofprospering</t>
+          <t>thehomelylondon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-15 11:53:04</t>
+          <t>2026-09-18 15:51:23</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@theartofprospering</t>
+          <t>https://www.tiktok.com/@thehomelylondon</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>syrashid</t>
+          <t>tifetito02</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -4588,58 +4588,58 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-11 12:35:39</t>
+          <t>2026-09-16 21:55:36</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@syrashid</t>
+          <t>https://www.tiktok.com/@tifetito02</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>themamadee</t>
+          <t>tixtok148</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-09-10 19:23:49</t>
+          <t>2026-09-19 18:20:29</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@themamadee</t>
+          <t>https://www.tiktok.com/@tixtok148</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>tixtok148</t>
+          <t>shazzbegum0</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -4651,29 +4651,29 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-09-19 18:20:29</t>
+          <t>2026-09-15 11:58:02</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tixtok148</t>
+          <t>https://www.tiktok.com/@shazzbegum0</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>tifetito02</t>
+          <t>shoni1984</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -4690,133 +4690,133 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-09-16 21:55:36</t>
+          <t>2026-09-10 08:20:01</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tifetito02</t>
+          <t>https://www.tiktok.com/@shoni1984</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>treeboyltd</t>
+          <t>uksaleshop</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-09-19 13:31:02</t>
+          <t>2026-09-16 15:22:03</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@treeboyltd</t>
+          <t>https://www.tiktok.com/@uksaleshop</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>su.k806</t>
+          <t>treeboyltd</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Shatavari 1300mg Extra Strength</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-09-17 20:34:02</t>
+          <t>2026-09-19 13:31:02</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@su.k806</t>
+          <t>https://www.tiktok.com/@treeboyltd</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>uksaleshop</t>
+          <t>user5251816210173</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-09-16 15:22:03</t>
+          <t>2026-09-15 20:13:06</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@uksaleshop</t>
+          <t>https://www.tiktok.com/@user5251816210173</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>unshoped</t>
+          <t>user13457g</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4826,24 +4826,24 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:04</t>
+          <t>2026-09-10 08:04:29</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@unshoped</t>
+          <t>https://www.tiktok.com/@user13457g</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>user5251816210173</t>
+          <t>user806865620814</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
@@ -4860,24 +4860,24 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-09-15 20:13:06</t>
+          <t>2026-09-20 17:13:54</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user5251816210173</t>
+          <t>https://www.tiktok.com/@user806865620814</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>user13457g</t>
+          <t>user8318338677754</t>
         </is>
       </c>
       <c r="B128" t="inlineStr"/>
@@ -4894,85 +4894,85 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-09-10 08:04:29</t>
+          <t>2026-09-16 23:49:09</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user13457g</t>
+          <t>https://www.tiktok.com/@user8318338677754</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>user8318338677754</t>
+          <t>user9199380</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-09-16 23:49:09</t>
+          <t>2026-09-08 15:02:55</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user8318338677754</t>
+          <t>https://www.tiktok.com/@user9199380</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>user9199380</t>
+          <t>user7271293811175</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-09-08 15:02:55</t>
+          <t>2026-09-11 08:42:27</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user9199380</t>
+          <t>https://www.tiktok.com/@user7271293811175</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -5013,7 +5013,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>user7271293811175</t>
+          <t>vera77524</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
@@ -5030,24 +5030,24 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-09-11 08:42:27</t>
+          <t>2026-09-09 07:38:35</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user7271293811175</t>
+          <t>https://www.tiktok.com/@vera77524</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>vera77524</t>
+          <t>yemi.bello3</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
@@ -5064,17 +5064,17 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-09 07:38:35</t>
+          <t>2026-09-17 07:22:35</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vera77524</t>
+          <t>https://www.tiktok.com/@yemi.bello3</t>
         </is>
       </c>
     </row>
@@ -5103,7 +5103,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -5149,7 +5149,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>yemi.bello3</t>
+          <t>yourfindz0</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
@@ -5166,24 +5166,24 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-09-17 07:22:35</t>
+          <t>2026-09-19 13:38:02</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@yemi.bello3</t>
+          <t>https://www.tiktok.com/@yourfindz0</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>yourfindz0</t>
+          <t>yvonne21197</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -5200,28 +5200,36 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-09-19 13:38:02</t>
+          <t>2026-09-16 22:41:43</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@yourfindz0</t>
+          <t>https://www.tiktok.com/@yvonne21197</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>yvonne21197</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
+          <t>zahidaparveen624</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>1K-5K</t>
+        </is>
+      </c>
       <c r="D138" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -5234,93 +5242,17 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-09-16 22:41:43</t>
+          <t>2026-09-11 13:42:26</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@yvonne21197</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>zahidaparveen624</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>1K-5K</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>Green Burner</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>2026-09-11 13:42:26</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H139" t="inlineStr">
-        <is>
           <t>https://www.tiktok.com/@zahidaparveen624</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>zubairianaz15</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>Ashwagandha Coffee</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Free sample from seller</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>2026-09-05 22:51:12</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="H140" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@zubairianaz15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-25 15:00
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:H164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1175,75 +1175,75 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bettyaddo398</t>
+          <t>bex_lifeafter40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-14 14:52:28</t>
+          <t>2026-09-17 15:30:23</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bettyaddo398</t>
+          <t>https://www.tiktok.com/@bex_lifeafter40</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bex_lifeafter40</t>
+          <t>bgee2345</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-17 15:30:23</t>
+          <t>2026-09-19 22:31:01</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bex_lifeafter40</t>
+          <t>https://www.tiktok.com/@bgee2345</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>bgee2345</t>
+          <t>a13dde</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1260,65 +1260,69 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-19 22:31:01</t>
+          <t>2026-09-14 08:25:14</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bgee2345</t>
+          <t>https://www.tiktok.com/@a13dde</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>chek_mi_shocase</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>akiatuconteh</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hibiscus</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-22 17:56:02</t>
+          <t>2026-09-09 07:32:58</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chek_mi_shocase</t>
+          <t>https://www.tiktok.com/@akiatuconteh</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>chloeeflynnx</t>
+          <t>ali.syed873</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1328,24 +1332,24 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-16 11:07:02</t>
+          <t>2026-09-17 03:47:33</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chloeeflynnx</t>
+          <t>https://www.tiktok.com/@ali.syed873</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ali.syed873</t>
+          <t>alemap9</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1362,17 +1366,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-17 03:47:33</t>
+          <t>2026-09-14 00:26:00</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ali.syed873</t>
+          <t>https://www.tiktok.com/@alemap9</t>
         </is>
       </c>
     </row>
@@ -1549,75 +1553,75 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>barbaraasiedu771</t>
+          <t>be__beauty1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-09 21:11:27</t>
+          <t>2026-09-08 17:18:23</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@barbaraasiedu771</t>
+          <t>https://www.tiktok.com/@be__beauty1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>be__beauty1</t>
+          <t>beauty20208</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-08 17:18:23</t>
+          <t>2026-09-18 19:31:55</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@be__beauty1</t>
+          <t>https://www.tiktok.com/@beauty20208</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>beauty20208</t>
+          <t>beemahempire</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1634,31 +1638,31 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-18 19:31:55</t>
+          <t>2026-09-15 11:52:03</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@beauty20208</t>
+          <t>https://www.tiktok.com/@beemahempire</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>beemahempire</t>
+          <t>bellasbeauty07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1668,31 +1672,31 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-15 11:52:03</t>
+          <t>2026-09-08 10:16:05</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@beemahempire</t>
+          <t>https://www.tiktok.com/@bellasbeauty07</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>bellasbeauty07</t>
+          <t>bettyaddo398</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1702,24 +1706,24 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-08 10:16:05</t>
+          <t>2026-09-14 14:52:28</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bellasbeauty07</t>
+          <t>https://www.tiktok.com/@bettyaddo398</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1sultan786</t>
+          <t>_dosah</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1736,7 +1740,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-21 10:45:04</t>
+          <t>2026-09-21 14:58:25</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1746,14 +1750,14 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@1sultan786</t>
+          <t>https://www.tiktok.com/@_dosah</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>a13dde</t>
+          <t>1sultan786</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1770,31 +1774,27 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-14 08:25:14</t>
+          <t>2026-09-21 10:45:04</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@a13dde</t>
+          <t>https://www.tiktok.com/@1sultan786</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>akiatuconteh</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
+          <t>dulal.miah2471</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
@@ -1808,24 +1808,24 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-09 07:32:58</t>
+          <t>2026-09-14 07:26:09</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@akiatuconteh</t>
+          <t>https://www.tiktok.com/@dulal.miah2471</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>alemap9</t>
+          <t>drantero_10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
@@ -1842,24 +1842,24 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-14 00:26:00</t>
+          <t>2026-09-17 14:48:32</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@alemap9</t>
+          <t>https://www.tiktok.com/@drantero_10</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>_dosah</t>
+          <t>donsnewchapter</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1876,65 +1876,65 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-21 14:58:25</t>
+          <t>2026-09-16 09:45:02</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@_dosah</t>
+          <t>https://www.tiktok.com/@donsnewchapter</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>dy7yobwohcu6</t>
+          <t>dollywithplaits73</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-18 21:30:44</t>
+          <t>2026-09-16 16:47:28</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dy7yobwohcu6</t>
+          <t>https://www.tiktok.com/@dollywithplaits73</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dulal.miah2471</t>
+          <t>dillytwinmum</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1944,24 +1944,24 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-14 07:26:09</t>
+          <t>2026-09-21 09:55:02</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dulal.miah2471</t>
+          <t>https://www.tiktok.com/@dillytwinmum</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>drantero_10</t>
+          <t>diane.docherty</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -1978,24 +1978,24 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-17 14:48:32</t>
+          <t>2026-09-15 09:50:59</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@drantero_10</t>
+          <t>https://www.tiktok.com/@diane.docherty</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>donsnewchapter</t>
+          <t>deckynla</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2012,31 +2012,31 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-16 09:45:02</t>
+          <t>2026-09-09 11:52:15</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@donsnewchapter</t>
+          <t>https://www.tiktok.com/@deckynla</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>dollywithplaits73</t>
+          <t>dailydealsuk03</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2046,31 +2046,31 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-16 16:47:28</t>
+          <t>2026-09-21 10:45:03</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dollywithplaits73</t>
+          <t>https://www.tiktok.com/@dailydealsuk03</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>dillytwinmum</t>
+          <t>courageous527</t>
         </is>
       </c>
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2080,160 +2080,160 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-21 09:55:02</t>
+          <t>2026-09-11 19:24:33</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dillytwinmum</t>
+          <t>https://www.tiktok.com/@courageous527</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>diane.docherty</t>
+          <t>climax.scenes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-15 09:50:59</t>
+          <t>2026-09-21 06:20:00</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@diane.docherty</t>
+          <t>https://www.tiktok.com/@climax.scenes</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>deckynla</t>
+          <t>claudia.claudia970</t>
         </is>
       </c>
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-09 11:52:15</t>
+          <t>2026-09-20 22:09:26</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@deckynla</t>
+          <t>https://www.tiktok.com/@claudia.claudia970</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>dailydealsuk03</t>
+          <t>clare.w4</t>
         </is>
       </c>
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-21 10:45:03</t>
+          <t>2026-09-10 14:06:31</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dailydealsuk03</t>
+          <t>https://www.tiktok.com/@clare.w4</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>dabrat1138</t>
+          <t>clairedipple66</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-10 01:03:04</t>
+          <t>2026-09-16 07:44:02</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dabrat1138</t>
+          <t>https://www.tiktok.com/@clairedipple66</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>courageous527</t>
+          <t>chucky692</t>
         </is>
       </c>
       <c r="B50" t="inlineStr"/>
@@ -2250,24 +2250,24 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-11 19:24:33</t>
+          <t>2026-09-15 07:29:48</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@courageous527</t>
+          <t>https://www.tiktok.com/@chucky692</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>climax.scenes</t>
+          <t>chloeeflynnx</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2279,36 +2279,36 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-09-21 06:20:00</t>
+          <t>2026-09-16 11:07:02</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@climax.scenes</t>
+          <t>https://www.tiktok.com/@chloeeflynnx</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>claudia.claudia970</t>
+          <t>chek_mi_shocase</t>
         </is>
       </c>
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Hibiscus</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2318,24 +2318,24 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-20 22:09:26</t>
+          <t>2026-09-22 17:56:02</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@claudia.claudia970</t>
+          <t>https://www.tiktok.com/@chek_mi_shocase</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>clare.w4</t>
+          <t>hrahmancookings</t>
         </is>
       </c>
       <c r="B53" t="inlineStr"/>
@@ -2352,31 +2352,31 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-10 14:06:31</t>
+          <t>2026-09-08 19:45:29</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@clare.w4</t>
+          <t>https://www.tiktok.com/@hrahmancookings</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>clairedipple66</t>
+          <t>hinas_beauty_buys</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2386,24 +2386,24 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-16 07:44:02</t>
+          <t>2026-09-18 09:46:05</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@clairedipple66</t>
+          <t>https://www.tiktok.com/@hinas_beauty_buys</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>chucky692</t>
+          <t>hchahal80</t>
         </is>
       </c>
       <c r="B55" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-15 07:29:48</t>
+          <t>2026-09-15 20:35:21</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2430,55 +2430,55 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@chucky692</t>
+          <t>https://www.tiktok.com/@hchahal80</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>i.couldnt.give.a.fuckkkk</t>
+          <t>hashirahmed784</t>
         </is>
       </c>
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-12 11:58:47</t>
+          <t>2026-09-21 21:16:02</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@i.couldnt.give.a.fuckkkk</t>
+          <t>https://www.tiktok.com/@hashirahmed784</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>hrahmancookings</t>
+          <t>jagjeetsinghkhals28</t>
         </is>
       </c>
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2488,99 +2488,99 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-08 19:45:29</t>
+          <t>2026-09-22 19:57:03</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hrahmancookings</t>
+          <t>https://www.tiktok.com/@jagjeetsinghkhals28</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>hinas_beauty_buys</t>
+          <t>i.couldnt.give.a.fuckkkk</t>
         </is>
       </c>
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-18 09:46:05</t>
+          <t>2026-09-12 11:58:47</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hinas_beauty_buys</t>
+          <t>https://www.tiktok.com/@i.couldnt.give.a.fuckkkk</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>hchahal80</t>
+          <t>janetaliciac</t>
         </is>
       </c>
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-15 20:35:21</t>
+          <t>2026-09-18 18:16:03</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hchahal80</t>
+          <t>https://www.tiktok.com/@janetaliciac</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>jagjeetsinghkhals28</t>
+          <t>dy7yobwohcu6</t>
         </is>
       </c>
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2590,58 +2590,58 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:03</t>
+          <t>2026-09-18 21:30:44</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@jagjeetsinghkhals28</t>
+          <t>https://www.tiktok.com/@dy7yobwohcu6</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>janetaliciac</t>
+          <t>gella4573</t>
         </is>
       </c>
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-18 18:16:03</t>
+          <t>2026-09-16 07:50:13</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@janetaliciac</t>
+          <t>https://www.tiktok.com/@gella4573</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>jem17363</t>
+          <t>georgiafergg</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -2658,41 +2658,41 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-09-21 17:28:16</t>
+          <t>2026-09-16 09:42:03</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@jem17363</t>
+          <t>https://www.tiktok.com/@georgiafergg</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>elizabethj27</t>
+          <t>gl80.31</t>
         </is>
       </c>
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-10 23:49:16</t>
+          <t>2026-09-10 23:30:20</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2702,21 +2702,21 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@elizabethj27</t>
+          <t>https://www.tiktok.com/@gl80.31</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>georgiafergg</t>
+          <t>haseeb.mum</t>
         </is>
       </c>
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2736,55 +2736,55 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@georgiafergg</t>
+          <t>https://www.tiktok.com/@haseeb.mum</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>gl80.31</t>
+          <t>emaanttshop</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-10 23:30:20</t>
+          <t>2026-09-15 21:32:02</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gl80.31</t>
+          <t>https://www.tiktok.com/@emaanttshop</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>haseeb.mum</t>
+          <t>eni_folabi</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2794,99 +2794,99 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-09-16 09:42:03</t>
+          <t>2026-09-09 11:38:46</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@haseeb.mum</t>
+          <t>https://www.tiktok.com/@eni_folabi</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>hashirahmed784</t>
+          <t>elizabetho001</t>
         </is>
       </c>
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-21 21:16:02</t>
+          <t>2026-09-08 17:27:54</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hashirahmed784</t>
+          <t>https://www.tiktok.com/@elizabetho001</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>eni_folabi</t>
+          <t>elizabethj27</t>
         </is>
       </c>
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-09 11:38:46</t>
+          <t>2026-09-10 23:49:16</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@eni_folabi</t>
+          <t>https://www.tiktok.com/@elizabethj27</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>feesdeals</t>
+          <t>kay.h0</t>
         </is>
       </c>
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2896,65 +2896,65 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-22 22:40:02</t>
+          <t>2026-09-09 04:27:35</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@feesdeals</t>
+          <t>https://www.tiktok.com/@kay.h0</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>elizabetho001</t>
+          <t>katseyelocer</t>
         </is>
       </c>
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-08 17:27:54</t>
+          <t>2026-09-15 22:58:52</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@elizabetho001</t>
+          <t>https://www.tiktok.com/@katseyelocer</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>emaanttshop</t>
+          <t>kaylee_dexter</t>
         </is>
       </c>
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2964,24 +2964,24 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-15 21:32:02</t>
+          <t>2026-09-22 19:57:02</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@emaanttshop</t>
+          <t>https://www.tiktok.com/@kaylee_dexter</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>kaylee_dexter</t>
+          <t>kayne202104</t>
         </is>
       </c>
       <c r="B72" t="inlineStr"/>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:02</t>
+          <t>2026-09-22 21:46:02</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3008,75 +3008,75 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kaylee_dexter</t>
+          <t>https://www.tiktok.com/@kayne202104</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>kay.h0</t>
+          <t>kennybabe692</t>
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-09 04:27:35</t>
+          <t>2026-09-10 11:43:02</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kay.h0</t>
+          <t>https://www.tiktok.com/@kennybabe692</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>kayne202104</t>
+          <t>kofoworola2853</t>
         </is>
       </c>
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-09-22 21:46:02</t>
+          <t>2026-09-11 10:52:59</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kayne202104</t>
+          <t>https://www.tiktok.com/@kofoworola2853</t>
         </is>
       </c>
     </row>
@@ -3117,14 +3117,14 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>kofoworola2853</t>
+          <t>keeskloset</t>
         </is>
       </c>
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3134,24 +3134,24 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-09-11 10:52:59</t>
+          <t>2026-09-16 09:57:04</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kofoworola2853</t>
+          <t>https://www.tiktok.com/@keeskloset</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>konaduroi</t>
+          <t>ladydonigbinosa</t>
         </is>
       </c>
       <c r="B77" t="inlineStr"/>
@@ -3168,31 +3168,31 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-15 03:00:44</t>
+          <t>2026-09-14 07:25:08</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@konaduroi</t>
+          <t>https://www.tiktok.com/@ladydonigbinosa</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>keeskloset</t>
+          <t>konaduroi</t>
         </is>
       </c>
       <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3202,31 +3202,31 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-16 09:57:04</t>
+          <t>2026-09-15 03:00:44</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@keeskloset</t>
+          <t>https://www.tiktok.com/@konaduroi</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>kennybabe692</t>
+          <t>leerobert123</t>
         </is>
       </c>
       <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3236,92 +3236,92 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-09-10 11:43:02</t>
+          <t>2026-09-22 19:57:02</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kennybabe692</t>
+          <t>https://www.tiktok.com/@leerobert123</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>leerobert123</t>
+          <t>life52551</t>
         </is>
       </c>
       <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:02</t>
+          <t>2026-09-21 22:10:02</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@leerobert123</t>
+          <t>https://www.tiktok.com/@life52551</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ladydonigbinosa</t>
+          <t>m.3384</t>
         </is>
       </c>
       <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-09-14 07:25:08</t>
+          <t>2026-09-21 10:22:24</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ladydonigbinosa</t>
+          <t>https://www.tiktok.com/@m.3384</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>life52551</t>
+          <t>lucia25070</t>
         </is>
       </c>
       <c r="B82" t="inlineStr"/>
@@ -3338,31 +3338,31 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-09-21 22:10:02</t>
+          <t>2026-09-18 09:46:03</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@life52551</t>
+          <t>https://www.tiktok.com/@lucia25070</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>lucia25070</t>
+          <t>maish1002</t>
         </is>
       </c>
       <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3372,92 +3372,92 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-18 09:46:03</t>
+          <t>2026-09-19 13:31:02</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@lucia25070</t>
+          <t>https://www.tiktok.com/@maish1002</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>maish1002</t>
+          <t>markh_8</t>
         </is>
       </c>
       <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-09-19 13:31:02</t>
+          <t>2026-09-09 16:07:49</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@maish1002</t>
+          <t>https://www.tiktok.com/@markh_8</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>m.3384</t>
+          <t>maxi_berrie</t>
         </is>
       </c>
       <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-09-21 10:22:24</t>
+          <t>2026-09-22 23:20:40</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@m.3384</t>
+          <t>https://www.tiktok.com/@maxi_berrie</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>markh_8</t>
+          <t>mehmoonaali238</t>
         </is>
       </c>
       <c r="B86" t="inlineStr"/>
@@ -3474,24 +3474,24 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-09-09 16:07:49</t>
+          <t>2026-09-17 11:42:05</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@markh_8</t>
+          <t>https://www.tiktok.com/@mehmoonaali238</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>maxi_berrie</t>
+          <t>merz3859</t>
         </is>
       </c>
       <c r="B87" t="inlineStr"/>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-09-22 23:20:40</t>
+          <t>2026-09-22 21:09:48</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3518,14 +3518,14 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@maxi_berrie</t>
+          <t>https://www.tiktok.com/@merz3859</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>mehmoonaali238</t>
+          <t>missyspranno12</t>
         </is>
       </c>
       <c r="B88" t="inlineStr"/>
@@ -3542,24 +3542,24 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-09-17 11:42:05</t>
+          <t>2026-09-15 13:31:44</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mehmoonaali238</t>
+          <t>https://www.tiktok.com/@missyspranno12</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>merz3859</t>
+          <t>monicalavern</t>
         </is>
       </c>
       <c r="B89" t="inlineStr"/>
@@ -3576,24 +3576,24 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-09-22 21:09:48</t>
+          <t>2026-09-15 13:00:13</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@merz3859</t>
+          <t>https://www.tiktok.com/@monicalavern</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>missyspranno12</t>
+          <t>moon19867</t>
         </is>
       </c>
       <c r="B90" t="inlineStr"/>
@@ -3610,24 +3610,24 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-09-15 13:31:44</t>
+          <t>2026-09-11 19:21:54</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@missyspranno12</t>
+          <t>https://www.tiktok.com/@moon19867</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>monicalavern</t>
+          <t>muhammadsha110</t>
         </is>
       </c>
       <c r="B91" t="inlineStr"/>
@@ -3644,24 +3644,24 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-09-15 13:00:13</t>
+          <t>2026-09-11 15:36:47</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@monicalavern</t>
+          <t>https://www.tiktok.com/@muhammadsha110</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>moon19867</t>
+          <t>jem17363</t>
         </is>
       </c>
       <c r="B92" t="inlineStr"/>
@@ -3678,24 +3678,24 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-09-11 19:21:54</t>
+          <t>2026-09-21 17:28:16</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@moon19867</t>
+          <t>https://www.tiktok.com/@jem17363</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>muhammadsha110</t>
+          <t>joandusabe</t>
         </is>
       </c>
       <c r="B93" t="inlineStr"/>
@@ -3712,58 +3712,58 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-09-11 15:36:47</t>
+          <t>2026-09-19 08:31:29</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@muhammadsha110</t>
+          <t>https://www.tiktok.com/@joandusabe</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>mymojomindset</t>
+          <t>journey2debtfree</t>
         </is>
       </c>
       <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-09-15 10:29:05</t>
+          <t>2026-09-22 19:57:02</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mymojomindset</t>
+          <t>https://www.tiktok.com/@journey2debtfree</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>joandusabe</t>
+          <t>julietogu5</t>
         </is>
       </c>
       <c r="B95" t="inlineStr"/>
@@ -3780,58 +3780,58 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-09-19 08:31:29</t>
+          <t>2026-09-14 01:42:26</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@joandusabe</t>
+          <t>https://www.tiktok.com/@julietogu5</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>journey2debtfree</t>
+          <t>jxnxxkxk</t>
         </is>
       </c>
       <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:02</t>
+          <t>2026-09-15 12:32:04</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@journey2debtfree</t>
+          <t>https://www.tiktok.com/@jxnxxkxk</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>julietogu5</t>
+          <t>k.tee146</t>
         </is>
       </c>
       <c r="B97" t="inlineStr"/>
@@ -3848,24 +3848,24 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-09-14 01:42:26</t>
+          <t>2026-09-10 09:41:07</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@julietogu5</t>
+          <t>https://www.tiktok.com/@k.tee146</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>jxnxxkxk</t>
+          <t>kamo76710</t>
         </is>
       </c>
       <c r="B98" t="inlineStr"/>
@@ -3882,58 +3882,58 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-09-15 12:32:04</t>
+          <t>2026-09-20 05:21:24</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@jxnxxkxk</t>
+          <t>https://www.tiktok.com/@kamo76710</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>k.tee146</t>
+          <t>feesdeals</t>
         </is>
       </c>
       <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-09-10 09:41:07</t>
+          <t>2026-09-22 22:40:02</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@k.tee146</t>
+          <t>https://www.tiktok.com/@feesdeals</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>kamo76710</t>
+          <t>fernandasprivy</t>
         </is>
       </c>
       <c r="B100" t="inlineStr"/>
@@ -3950,24 +3950,24 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-20 05:21:24</t>
+          <t>2026-09-15 19:00:52</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kamo76710</t>
+          <t>https://www.tiktok.com/@fernandasprivy</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>katseyelocer</t>
+          <t>oluwatoyosiabayom</t>
         </is>
       </c>
       <c r="B101" t="inlineStr"/>
@@ -3984,31 +3984,39 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-09-15 22:58:52</t>
+          <t>2026-09-14 17:04:02</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@katseyelocer</t>
+          <t>https://www.tiktok.com/@oluwatoyosiabayom</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>fernandasprivy</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
+          <t>olascornerpage</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>1K-5K</t>
+        </is>
+      </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -4018,65 +4026,65 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-09-15 19:00:52</t>
+          <t>2026-09-12 21:52:02</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fernandasprivy</t>
+          <t>https://www.tiktok.com/@olascornerpage</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>gella4573</t>
+          <t>oladayomartins</t>
         </is>
       </c>
       <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-09-16 07:50:13</t>
+          <t>2026-09-17 21:17:16</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gella4573</t>
+          <t>https://www.tiktok.com/@oladayomartins</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>omolade.abebi</t>
+          <t>nxthxnfrxmdxy</t>
         </is>
       </c>
       <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -4086,73 +4094,65 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-17 10:33:35</t>
+          <t>2026-09-22 19:57:02</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@omolade.abebi</t>
+          <t>https://www.tiktok.com/@nxthxnfrxmdxy</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>oluwatoyosiabayom</t>
+          <t>nrahi28</t>
         </is>
       </c>
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-14 17:04:02</t>
+          <t>2026-09-20 14:59:29</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oluwatoyosiabayom</t>
+          <t>https://www.tiktok.com/@nrahi28</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>olascornerpage</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>1K-5K</t>
-        </is>
-      </c>
+          <t>nancymm52</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4162,65 +4162,65 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-12 21:52:02</t>
+          <t>2026-09-18 07:04:23</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@olascornerpage</t>
+          <t>https://www.tiktok.com/@nancymm52</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>oladayomartins</t>
+          <t>nanahdaramy</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-17 21:17:16</t>
+          <t>2026-09-14 00:12:20</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oladayomartins</t>
+          <t>https://www.tiktok.com/@nanahdaramy</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>nxthxnfrxmdxy</t>
+          <t>na2706_1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -4230,24 +4230,24 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:02</t>
+          <t>2026-09-20 23:38:18</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nxthxnfrxmdxy</t>
+          <t>https://www.tiktok.com/@na2706_1</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>nrahi28</t>
+          <t>mymojomindset</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -4264,24 +4264,24 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-20 14:59:29</t>
+          <t>2026-09-15 10:29:05</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nrahi28</t>
+          <t>https://www.tiktok.com/@mymojomindset</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>nancymm52</t>
+          <t>queeen_0f_hearts</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -4298,24 +4298,24 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-18 07:04:23</t>
+          <t>2026-09-13 23:51:38</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nancymm52</t>
+          <t>https://www.tiktok.com/@queeen_0f_hearts</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>nanahdaramy</t>
+          <t>positivevibeonly62</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -4332,24 +4332,24 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-14 00:12:20</t>
+          <t>2026-09-21 10:52:02</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nanahdaramy</t>
+          <t>https://www.tiktok.com/@positivevibeonly62</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>na2706_1</t>
+          <t>radhekrishna_11</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -4366,17 +4366,17 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-20 23:38:18</t>
+          <t>2026-09-21 11:21:47</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@na2706_1</t>
+          <t>https://www.tiktok.com/@radhekrishna_11</t>
         </is>
       </c>
     </row>
@@ -4417,14 +4417,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>queeen_0f_hearts</t>
+          <t>online.shop8292</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4434,24 +4434,24 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-09-13 23:51:38</t>
+          <t>2026-09-22 19:57:03</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@queeen_0f_hearts</t>
+          <t>https://www.tiktok.com/@online.shop8292</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ranifarooq_3</t>
+          <t>positiveproductsuk</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -4463,29 +4463,29 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-09-13 22:37:56</t>
+          <t>2026-09-15 11:53:04</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ranifarooq_3</t>
+          <t>https://www.tiktok.com/@positiveproductsuk</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>radhekrishna_11</t>
+          <t>omolade.abebi</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -4502,24 +4502,24 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-21 11:21:47</t>
+          <t>2026-09-17 10:33:35</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@radhekrishna_11</t>
+          <t>https://www.tiktok.com/@omolade.abebi</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>oyetunji.sunday</t>
+          <t>rozana2026</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -4536,65 +4536,65 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-12 13:08:25</t>
+          <t>2026-09-19 15:08:34</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oyetunji.sunday</t>
+          <t>https://www.tiktok.com/@rozana2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>positivevibeonly62</t>
+          <t>rory.the.cocker</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-21 10:52:02</t>
+          <t>2026-09-18 18:13:02</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@positivevibeonly62</t>
+          <t>https://www.tiktok.com/@rory.the.cocker</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>online.shop8292</t>
+          <t>ruksi1607</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -4604,24 +4604,24 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:03</t>
+          <t>2026-09-13 20:49:20</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@online.shop8292</t>
+          <t>https://www.tiktok.com/@ruksi1607</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ruksi1607</t>
+          <t>saadia7166</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -4638,58 +4638,58 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-09-13 20:49:20</t>
+          <t>2026-09-10 11:16:51</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ruksi1607</t>
+          <t>https://www.tiktok.com/@saadia7166</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>rozana2026</t>
+          <t>sbegum.79</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-09-19 15:08:34</t>
+          <t>2026-09-21 17:38:25</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rozana2026</t>
+          <t>https://www.tiktok.com/@sbegum.79</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>saadia7166</t>
+          <t>sedi546</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -4706,17 +4706,17 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-09-10 11:16:51</t>
+          <t>2026-09-13 15:46:07</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@saadia7166</t>
+          <t>https://www.tiktok.com/@sedi546</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>sedi546</t>
+          <t>samirakarim24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr"/>
@@ -4774,41 +4774,41 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-09-13 15:46:07</t>
+          <t>2026-09-11 11:10:48</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sedi546</t>
+          <t>https://www.tiktok.com/@samirakarim24</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>seffshops</t>
+          <t>sehnamiee</t>
         </is>
       </c>
       <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-09-21 10:52:04</t>
+          <t>2026-09-21 20:46:02</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -4818,21 +4818,21 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@seffshops</t>
+          <t>https://www.tiktok.com/@sehnamiee</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>samirakarim24</t>
+          <t>seffshops</t>
         </is>
       </c>
       <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -4842,51 +4842,51 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-09-11 11:10:48</t>
+          <t>2026-09-21 10:52:04</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@samirakarim24</t>
+          <t>https://www.tiktok.com/@seffshops</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>sbegum.79</t>
+          <t>sexybaby7657</t>
         </is>
       </c>
       <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-09-21 17:38:25</t>
+          <t>2026-09-09 21:00:27</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sbegum.79</t>
+          <t>https://www.tiktok.com/@sexybaby7657</t>
         </is>
       </c>
     </row>
@@ -4927,41 +4927,41 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>sehnamiee</t>
+          <t>reems_ttsshop</t>
         </is>
       </c>
       <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-09-21 20:46:02</t>
+          <t>2026-09-22 19:57:02</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sehnamiee</t>
+          <t>https://www.tiktok.com/@reems_ttsshop</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>shazzbegum0</t>
+          <t>ranifarooq_3</t>
         </is>
       </c>
       <c r="B130" t="inlineStr"/>
@@ -4973,29 +4973,29 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-09-15 11:58:02</t>
+          <t>2026-09-13 22:37:56</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shazzbegum0</t>
+          <t>https://www.tiktok.com/@ranifarooq_3</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>sexybaby7657</t>
+          <t>oyetunji.sunday</t>
         </is>
       </c>
       <c r="B131" t="inlineStr"/>
@@ -5012,31 +5012,31 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-09-09 21:00:27</t>
+          <t>2026-09-12 13:08:25</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sexybaby7657</t>
+          <t>https://www.tiktok.com/@oyetunji.sunday</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>reems_ttsshop</t>
+          <t>padnerkupakuwana</t>
         </is>
       </c>
       <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5046,58 +5046,58 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:02</t>
+          <t>2026-09-13 02:02:06</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@reems_ttsshop</t>
+          <t>https://www.tiktok.com/@padnerkupakuwana</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>rory.the.cocker</t>
+          <t>sjahan83</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-18 18:13:02</t>
+          <t>2026-09-12 13:46:48</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rory.the.cocker</t>
+          <t>https://www.tiktok.com/@sjahan83</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>padnerkupakuwana</t>
+          <t>shukar7860</t>
         </is>
       </c>
       <c r="B134" t="inlineStr"/>
@@ -5114,31 +5114,31 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-09-13 02:02:06</t>
+          <t>2026-09-22 09:29:34</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@padnerkupakuwana</t>
+          <t>https://www.tiktok.com/@shukar7860</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>positiveproductsuk</t>
+          <t>shopforfiver</t>
         </is>
       </c>
       <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5148,24 +5148,24 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-09-15 11:53:04</t>
+          <t>2026-09-21 15:01:03</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@positiveproductsuk</t>
+          <t>https://www.tiktok.com/@shopforfiver</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>sjahan83</t>
+          <t>shoni1984</t>
         </is>
       </c>
       <c r="B136" t="inlineStr"/>
@@ -5182,24 +5182,24 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-09-12 13:46:48</t>
+          <t>2026-09-10 08:20:01</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sjahan83</t>
+          <t>https://www.tiktok.com/@shoni1984</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>shukar7860</t>
+          <t>syrashid</t>
         </is>
       </c>
       <c r="B137" t="inlineStr"/>
@@ -5216,92 +5216,92 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-09-22 09:29:34</t>
+          <t>2026-09-11 12:35:39</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shukar7860</t>
+          <t>https://www.tiktok.com/@syrashid</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>shopforfiver</t>
+          <t>thehomelylondon</t>
         </is>
       </c>
       <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-09-21 15:01:03</t>
+          <t>2026-09-18 15:51:23</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shopforfiver</t>
+          <t>https://www.tiktok.com/@thehomelylondon</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>shoni1984</t>
+          <t>steffispicks</t>
         </is>
       </c>
       <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Spearmint</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-09-10 08:20:01</t>
+          <t>2026-09-22 19:57:03</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shoni1984</t>
+          <t>https://www.tiktok.com/@steffispicks</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>syrashid</t>
+          <t>ste.baby6</t>
         </is>
       </c>
       <c r="B140" t="inlineStr"/>
@@ -5318,92 +5318,92 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-09-11 12:35:39</t>
+          <t>2026-09-09 16:28:17</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@syrashid</t>
+          <t>https://www.tiktok.com/@ste.baby6</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>thehomelylondon</t>
+          <t>tifetito02</t>
         </is>
       </c>
       <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-09-18 15:51:23</t>
+          <t>2026-09-16 21:55:36</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@thehomelylondon</t>
+          <t>https://www.tiktok.com/@tifetito02</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>steffispicks</t>
+          <t>themamadee</t>
         </is>
       </c>
       <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Spearmint</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:03</t>
+          <t>2026-09-10 19:23:49</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@steffispicks</t>
+          <t>https://www.tiktok.com/@themamadee</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ste.baby6</t>
+          <t>trendtokshop88</t>
         </is>
       </c>
       <c r="B143" t="inlineStr"/>
@@ -5420,58 +5420,58 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-09-09 16:28:17</t>
+          <t>2026-09-22 19:57:03</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ste.baby6</t>
+          <t>https://www.tiktok.com/@trendtokshop88</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>tifetito02</t>
+          <t>tixtok148</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-09-16 21:55:36</t>
+          <t>2026-09-19 18:20:29</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tifetito02</t>
+          <t>https://www.tiktok.com/@tixtok148</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>themamadee</t>
+          <t>tyanie1703</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -5488,160 +5488,160 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-09-10 19:23:49</t>
+          <t>2026-09-22 14:51:38</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@themamadee</t>
+          <t>https://www.tiktok.com/@tyanie1703</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>trendtokshop88</t>
+          <t>uksaleshop</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-09-22 19:57:03</t>
+          <t>2026-09-16 15:22:03</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@trendtokshop88</t>
+          <t>https://www.tiktok.com/@uksaleshop</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>tixtok148</t>
+          <t>user13457g</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-09-19 18:20:29</t>
+          <t>2026-09-10 08:04:29</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tixtok148</t>
+          <t>https://www.tiktok.com/@user13457g</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>tyanie1703</t>
+          <t>su.k806</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Shatavari 1300mg Extra Strength</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-09-22 14:51:38</t>
+          <t>2026-09-17 20:34:02</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tyanie1703</t>
+          <t>https://www.tiktok.com/@su.k806</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>uksaleshop</t>
+          <t>user2182373993526</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-09-16 15:22:03</t>
+          <t>2026-09-21 12:26:17</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@uksaleshop</t>
+          <t>https://www.tiktok.com/@user2182373993526</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>user13457g</t>
+          <t>user2773140226152</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -5658,58 +5658,58 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-09-10 08:04:29</t>
+          <t>2026-09-21 20:00:10</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user13457g</t>
+          <t>https://www.tiktok.com/@user2773140226152</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>su.k806</t>
+          <t>user7271293811175</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Shatavari 1300mg Extra Strength</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-09-17 20:34:02</t>
+          <t>2026-09-11 08:42:27</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@su.k806</t>
+          <t>https://www.tiktok.com/@user7271293811175</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>user2182373993526</t>
+          <t>user5251816210173</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -5726,24 +5726,24 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-09-21 12:26:17</t>
+          <t>2026-09-15 20:13:06</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user2182373993526</t>
+          <t>https://www.tiktok.com/@user5251816210173</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>user2773140226152</t>
+          <t>user8318338677754</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -5760,92 +5760,92 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-09-21 20:00:10</t>
+          <t>2026-09-16 23:49:09</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user2773140226152</t>
+          <t>https://www.tiktok.com/@user8318338677754</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>user7271293811175</t>
+          <t>user9199380</t>
         </is>
       </c>
       <c r="B154" t="inlineStr"/>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-09-11 08:42:27</t>
+          <t>2026-09-08 15:02:55</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user7271293811175</t>
+          <t>https://www.tiktok.com/@user9199380</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>user5251816210173</t>
+          <t>user_78602223</t>
         </is>
       </c>
       <c r="B155" t="inlineStr"/>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-09-15 20:13:06</t>
+          <t>2026-09-22 17:40:46</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user5251816210173</t>
+          <t>https://www.tiktok.com/@user_78602223</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>user8318338677754</t>
+          <t>user806865620814</t>
         </is>
       </c>
       <c r="B156" t="inlineStr"/>
@@ -5862,92 +5862,92 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-09-16 23:49:09</t>
+          <t>2026-09-20 17:13:54</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user8318338677754</t>
+          <t>https://www.tiktok.com/@user806865620814</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>user9199380</t>
+          <t>vain119</t>
         </is>
       </c>
       <c r="B157" t="inlineStr"/>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-09-08 15:02:55</t>
+          <t>2026-09-15 09:25:05</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user9199380</t>
+          <t>https://www.tiktok.com/@vain119</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>user_78602223</t>
+          <t>vera77524</t>
         </is>
       </c>
       <c r="B158" t="inlineStr"/>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-09-22 17:40:46</t>
+          <t>2026-09-09 07:38:35</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user_78602223</t>
+          <t>https://www.tiktok.com/@vera77524</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>user806865620814</t>
+          <t>yemi.bello3</t>
         </is>
       </c>
       <c r="B159" t="inlineStr"/>
@@ -5964,58 +5964,58 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>2026-09-20 17:13:54</t>
+          <t>2026-09-17 07:22:35</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user806865620814</t>
+          <t>https://www.tiktok.com/@yemi.bello3</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>vain119</t>
+          <t>vikingbeardshop</t>
         </is>
       </c>
       <c r="B160" t="inlineStr"/>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Shatavari 1300mg Extra Strength</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-09-15 09:25:05</t>
+          <t>2026-09-19 13:38:02</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vain119</t>
+          <t>https://www.tiktok.com/@vikingbeardshop</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>vera77524</t>
+          <t>yemishittuedemayibo</t>
         </is>
       </c>
       <c r="B161" t="inlineStr"/>
@@ -6032,24 +6032,24 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-09-09 07:38:35</t>
+          <t>2026-09-19 00:15:14</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vera77524</t>
+          <t>https://www.tiktok.com/@yemishittuedemayibo</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>yemi.bello3</t>
+          <t>yourfindz0</t>
         </is>
       </c>
       <c r="B162" t="inlineStr"/>
@@ -6066,62 +6066,70 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2026-09-17 07:22:35</t>
+          <t>2026-09-19 13:38:02</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@yemi.bello3</t>
+          <t>https://www.tiktok.com/@yourfindz0</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>vikingbeardshop</t>
+          <t>yvonne21197</t>
         </is>
       </c>
       <c r="B163" t="inlineStr"/>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Shatavari 1300mg Extra Strength</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>2026-09-19 13:38:02</t>
+          <t>2026-09-16 22:41:43</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vikingbeardshop</t>
+          <t>https://www.tiktok.com/@yvonne21197</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>yemishittuedemayibo</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr"/>
-      <c r="C164" t="inlineStr"/>
+          <t>zahidaparveen624</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>1K-5K</t>
+        </is>
+      </c>
       <c r="D164" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -6134,125 +6142,15 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>2026-09-19 00:15:14</t>
+          <t>2026-09-11 13:42:26</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@yemishittuedemayibo</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>yourfindz0</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr"/>
-      <c r="C165" t="inlineStr"/>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Green Burner</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>2026-09-19 13:38:02</t>
-        </is>
-      </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@yourfindz0</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>yvonne21197</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr"/>
-      <c r="C166" t="inlineStr"/>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Green Burner</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
-        </is>
-      </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>2026-09-16 22:41:43</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@yvonne21197</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>zahidaparveen624</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>1K-5K</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Green Burner</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>2026-09-11 13:42:26</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@zahidaparveen624</t>
         </is>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-01 13:07
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -6207,7 +6207,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-13 15:39
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H247"/>
+  <dimension ref="A1:H248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -691,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4523,7 +4523,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>louisesoutar44</t>
+          <t>smartfindsuk1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4533,12 +4533,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>1K-5K</t>
+          <t>0-1K</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4548,24 +4548,24 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-10-06 12:41:03</t>
+          <t>2026-10-01 10:48:02</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@louisesoutar44</t>
+          <t>https://www.tiktok.com/@smartfindsuk1</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>smartfindsuk1</t>
+          <t>louisesoutar44</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4575,12 +4575,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>0-1K</t>
+          <t>1K-5K</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4590,17 +4590,17 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-10-01 10:48:02</t>
+          <t>2026-10-06 12:41:03</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@smartfindsuk1</t>
+          <t>https://www.tiktok.com/@louisesoutar44</t>
         </is>
       </c>
     </row>
@@ -6367,75 +6367,83 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>kaz.gym82</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
+          <t>shopwithsk19</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>0-1K</t>
+        </is>
+      </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-10-05 08:29:56</t>
+          <t>2026-10-07 11:56:02</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kaz.gym82</t>
+          <t>https://www.tiktok.com/@shopwithsk19</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>isinfaye456</t>
+          <t>juliana_armoh</t>
         </is>
       </c>
       <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-10-06 14:00:36</t>
+          <t>2026-10-01 21:22:31</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@isinfaye456</t>
+          <t>https://www.tiktok.com/@juliana_armoh</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ilzb7</t>
+          <t>isinfaye456</t>
         </is>
       </c>
       <c r="B145" t="inlineStr"/>
@@ -6447,29 +6455,29 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-10-05 16:59:43</t>
+          <t>2026-10-06 14:00:36</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ilzb7</t>
+          <t>https://www.tiktok.com/@isinfaye456</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>idrissasesay7</t>
+          <t>ilzb7</t>
         </is>
       </c>
       <c r="B146" t="inlineStr"/>
@@ -6481,70 +6489,70 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-10-02 23:30:18</t>
+          <t>2026-10-05 16:59:43</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@idrissasesay7</t>
+          <t>https://www.tiktok.com/@ilzb7</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>gemfinds10</t>
+          <t>idrissasesay7</t>
         </is>
       </c>
       <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-10-11 17:36:02</t>
+          <t>2026-10-02 23:30:18</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gemfinds10</t>
+          <t>https://www.tiktok.com/@idrissasesay7</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>katelisterx</t>
+          <t>gemfinds10</t>
         </is>
       </c>
       <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
-          <t>[Advent Calendar] 2026</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6554,7 +6562,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-10-11 13:16:02</t>
+          <t>2026-10-11 17:36:02</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -6564,21 +6572,21 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@katelisterx</t>
+          <t>https://www.tiktok.com/@gemfinds10</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>juliana_armoh</t>
+          <t>kates_space_11.11</t>
         </is>
       </c>
       <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6588,24 +6596,24 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-10-01 21:22:31</t>
+          <t>2026-10-11 17:31:03</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@juliana_armoh</t>
+          <t>https://www.tiktok.com/@kates_space_11.11</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>kates_space_11.11</t>
+          <t>katelisterx</t>
         </is>
       </c>
       <c r="B150" t="inlineStr"/>
@@ -6622,7 +6630,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-10-11 17:31:03</t>
+          <t>2026-10-11 13:16:02</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -6632,14 +6640,14 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kates_space_11.11</t>
+          <t>https://www.tiktok.com/@katelisterx</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>jean.makin</t>
+          <t>kennyshekoni</t>
         </is>
       </c>
       <c r="B151" t="inlineStr"/>
@@ -6651,29 +6659,29 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-10-03 14:41:36</t>
+          <t>2026-10-01 19:41:15</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@jean.makin</t>
+          <t>https://www.tiktok.com/@kennyshekoni</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>armaan.ahmed37</t>
+          <t>jean.makin</t>
         </is>
       </c>
       <c r="B152" t="inlineStr"/>
@@ -6690,7 +6698,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-10-03 19:49:39</t>
+          <t>2026-10-03 14:41:36</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6700,14 +6708,14 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@armaan.ahmed37</t>
+          <t>https://www.tiktok.com/@jean.makin</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>angelhairstylist1</t>
+          <t>armaan.ahmed37</t>
         </is>
       </c>
       <c r="B153" t="inlineStr"/>
@@ -6724,24 +6732,24 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-10-04 20:43:03</t>
+          <t>2026-10-03 19:49:39</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@angelhairstylist1</t>
+          <t>https://www.tiktok.com/@armaan.ahmed37</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>amena.akter3665</t>
+          <t>angelhairstylist1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr"/>
@@ -6753,36 +6761,36 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-09-28 12:23:28</t>
+          <t>2026-10-04 20:43:03</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@amena.akter3665</t>
+          <t>https://www.tiktok.com/@angelhairstylist1</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>amieuka</t>
+          <t>amena.akter3665</t>
         </is>
       </c>
       <c r="B155" t="inlineStr"/>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -6792,70 +6800,70 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-10-11 09:01:43</t>
+          <t>2026-09-28 12:23:28</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@amieuka</t>
+          <t>https://www.tiktok.com/@amena.akter3665</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>amap000</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>1K-5K</t>
-        </is>
-      </c>
+          <t>amieuka</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-10-03 10:59:49</t>
+          <t>2026-10-11 09:01:43</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@amap000</t>
+          <t>https://www.tiktok.com/@amieuka</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>bangladesh_216</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
+          <t>amap000</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>1K-5K</t>
+        </is>
+      </c>
       <c r="D157" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -6863,36 +6871,36 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-10-07 23:21:07</t>
+          <t>2026-10-03 10:59:49</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bangladesh_216</t>
+          <t>https://www.tiktok.com/@amap000</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>bestproducts12113</t>
+          <t>bangladesh_216</t>
         </is>
       </c>
       <c r="B158" t="inlineStr"/>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -6902,17 +6910,17 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-10-11 17:45:02</t>
+          <t>2026-10-07 23:21:07</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bestproducts12113</t>
+          <t>https://www.tiktok.com/@bangladesh_216</t>
         </is>
       </c>
     </row>
@@ -6953,14 +6961,14 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>bosetracysalvador</t>
+          <t>bestproducts12113</t>
         </is>
       </c>
       <c r="B160" t="inlineStr"/>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
@@ -6970,36 +6978,28 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-10-09 13:31:54</t>
+          <t>2026-10-11 17:45:02</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bosetracysalvador</t>
+          <t>https://www.tiktok.com/@bestproducts12113</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>_mohlad</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>0-1K</t>
-        </is>
-      </c>
+          <t>bukky.yoyo</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr"/>
+      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -7012,7 +7012,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-10-04 18:10:30</t>
+          <t>2026-10-04 16:50:32</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -7022,18 +7022,26 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@_mohlad</t>
+          <t>https://www.tiktok.com/@bukky.yoyo</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>adeede1</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr"/>
-      <c r="C162" t="inlineStr"/>
+          <t>_mohlad</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>0-1K</t>
+        </is>
+      </c>
       <c r="D162" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -7041,29 +7049,29 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2026-10-03 06:37:25</t>
+          <t>2026-10-04 18:10:30</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@adeede1</t>
+          <t>https://www.tiktok.com/@_mohlad</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>africanmotherxo</t>
+          <t>adeede1</t>
         </is>
       </c>
       <c r="B163" t="inlineStr"/>
@@ -7080,65 +7088,65 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>2026-10-07 22:50:15</t>
+          <t>2026-10-03 06:37:25</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@africanmotherxo</t>
+          <t>https://www.tiktok.com/@adeede1</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>hannah99r</t>
+          <t>africanmotherxo</t>
         </is>
       </c>
       <c r="B164" t="inlineStr"/>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
-          <t>[Advent Calendar] 2026</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>2026-10-11 17:31:03</t>
+          <t>2026-10-07 22:50:15</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hannah99r</t>
+          <t>https://www.tiktok.com/@africanmotherxo</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>hair.vendor.in.uk</t>
+          <t>hannah99r</t>
         </is>
       </c>
       <c r="B165" t="inlineStr"/>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
@@ -7148,58 +7156,58 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>2026-10-06 19:19:06</t>
+          <t>2026-10-11 17:31:03</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hair.vendor.in.uk</t>
+          <t>https://www.tiktok.com/@hannah99r</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>helenm566</t>
+          <t>hair.vendor.in.uk</t>
         </is>
       </c>
       <c r="B166" t="inlineStr"/>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-10-08 17:13:34</t>
+          <t>2026-10-06 19:19:06</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@helenm566</t>
+          <t>https://www.tiktok.com/@hair.vendor.in.uk</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>hu123342425</t>
+          <t>helenm566</t>
         </is>
       </c>
       <c r="B167" t="inlineStr"/>
@@ -7211,29 +7219,29 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>2026-10-04 15:47:04</t>
+          <t>2026-10-08 17:13:34</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@hu123342425</t>
+          <t>https://www.tiktok.com/@helenm566</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>don.forich</t>
+          <t>hu123342425</t>
         </is>
       </c>
       <c r="B168" t="inlineStr"/>
@@ -7245,36 +7253,36 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>2026-10-08 12:58:36</t>
+          <t>2026-10-04 15:47:04</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@don.forich</t>
+          <t>https://www.tiktok.com/@hu123342425</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>fastrunner1563</t>
+          <t>don.forich</t>
         </is>
       </c>
       <c r="B169" t="inlineStr"/>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
@@ -7284,17 +7292,17 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>2026-10-10 09:02:03</t>
+          <t>2026-10-08 12:58:36</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fastrunner1563</t>
+          <t>https://www.tiktok.com/@don.forich</t>
         </is>
       </c>
     </row>
@@ -7335,14 +7343,14 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>explorewithmex10</t>
+          <t>fastrunner1563</t>
         </is>
       </c>
       <c r="B171" t="inlineStr"/>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -7352,28 +7360,36 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2026-10-02 09:06:56</t>
+          <t>2026-10-10 09:02:03</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@explorewithmex10</t>
+          <t>https://www.tiktok.com/@fastrunner1563</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>dsda0786</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr"/>
-      <c r="C172" t="inlineStr"/>
+          <t>dontus05</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>£0-£50</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>5K-10K</t>
+        </is>
+      </c>
       <c r="D172" t="inlineStr">
         <is>
           <t>Green Burner</t>
@@ -7386,93 +7402,85 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>2026-09-29 09:46:30</t>
+          <t>2026-10-09 12:40:03</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dsda0786</t>
+          <t>https://www.tiktok.com/@dontus05</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>dontus05</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>£0-£50</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>5K-10K</t>
-        </is>
-      </c>
+          <t>duaanoor080120</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr"/>
+      <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>2026-10-09 12:40:03</t>
+          <t>2026-10-02 06:26:32</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dontus05</t>
+          <t>https://www.tiktok.com/@duaanoor080120</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>duaanoor080120</t>
+          <t>dsda0786</t>
         </is>
       </c>
       <c r="B174" t="inlineStr"/>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2026-10-02 06:26:32</t>
+          <t>2026-09-29 09:46:30</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@duaanoor080120</t>
+          <t>https://www.tiktok.com/@dsda0786</t>
         </is>
       </c>
     </row>
@@ -7547,14 +7555,14 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>biancaaaaenach</t>
+          <t>explorewithmex10</t>
         </is>
       </c>
       <c r="B177" t="inlineStr"/>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
@@ -7564,85 +7572,85 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>2026-10-09 12:10:04</t>
+          <t>2026-10-02 09:06:56</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@biancaaaaenach</t>
+          <t>https://www.tiktok.com/@explorewithmex10</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>caradanielleeats</t>
+          <t>bosetracysalvador</t>
         </is>
       </c>
       <c r="B178" t="inlineStr"/>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
-          <t>[Advent Calendar] 2026</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>2026-10-11 13:14:02</t>
+          <t>2026-10-09 13:31:54</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@caradanielleeats</t>
+          <t>https://www.tiktok.com/@bosetracysalvador</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>bukky.yoyo</t>
+          <t>biancaaaaenach</t>
         </is>
       </c>
       <c r="B179" t="inlineStr"/>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>2026-10-04 16:50:32</t>
+          <t>2026-10-09 12:10:04</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bukky.yoyo</t>
+          <t>https://www.tiktok.com/@biancaaaaenach</t>
         </is>
       </c>
     </row>
@@ -7683,14 +7691,14 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>damsel755</t>
+          <t>caradanielleeats</t>
         </is>
       </c>
       <c r="B181" t="inlineStr"/>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
@@ -7700,24 +7708,24 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>2026-10-05 20:02:55</t>
+          <t>2026-10-11 13:14:02</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@damsel755</t>
+          <t>https://www.tiktok.com/@caradanielleeats</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>dearlola45</t>
+          <t>damsel755</t>
         </is>
       </c>
       <c r="B182" t="inlineStr"/>
@@ -7734,58 +7742,58 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>2026-10-01 11:28:54</t>
+          <t>2026-10-05 20:02:55</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@dearlola45</t>
+          <t>https://www.tiktok.com/@damsel755</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>desylviaa1</t>
+          <t>dearlola45</t>
         </is>
       </c>
       <c r="B183" t="inlineStr"/>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>2026-09-27 10:40:10</t>
+          <t>2026-10-01 11:28:54</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@desylviaa1</t>
+          <t>https://www.tiktok.com/@dearlola45</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>kulwinderrani5</t>
+          <t>desylviaa1</t>
         </is>
       </c>
       <c r="B184" t="inlineStr"/>
@@ -7797,29 +7805,29 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2026-10-05 09:00:08</t>
+          <t>2026-09-27 10:40:10</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kulwinderrani5</t>
+          <t>https://www.tiktok.com/@desylviaa1</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>knicksmakeuppro</t>
+          <t>kulwinderrani5</t>
         </is>
       </c>
       <c r="B185" t="inlineStr"/>
@@ -7831,29 +7839,29 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>2026-10-01 11:30:23</t>
+          <t>2026-10-05 09:00:08</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@knicksmakeuppro</t>
+          <t>https://www.tiktok.com/@kulwinderrani5</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>kennyshekoni</t>
+          <t>knicksmakeuppro</t>
         </is>
       </c>
       <c r="B186" t="inlineStr"/>
@@ -7870,7 +7878,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2026-10-01 19:41:15</t>
+          <t>2026-10-01 11:30:23</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -7880,48 +7888,48 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@kennyshekoni</t>
+          <t>https://www.tiktok.com/@knicksmakeuppro</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>rks_m</t>
+          <t>kaz.gym82</t>
         </is>
       </c>
       <c r="B187" t="inlineStr"/>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-10-11 19:01:51</t>
+          <t>2026-10-05 08:29:56</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rks_m</t>
+          <t>https://www.tiktok.com/@kaz.gym82</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>saintmary.sobo</t>
+          <t>rtamakter</t>
         </is>
       </c>
       <c r="B188" t="inlineStr"/>
@@ -7938,24 +7946,24 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>2026-10-07 19:00:51</t>
+          <t>2026-10-05 22:45:22</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@saintmary.sobo</t>
+          <t>https://www.tiktok.com/@rtamakter</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ruas_dream</t>
+          <t>saintmary.sobo</t>
         </is>
       </c>
       <c r="B189" t="inlineStr"/>
@@ -7972,24 +7980,24 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>2026-09-27 11:00:34</t>
+          <t>2026-10-07 19:00:51</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ruas_dream</t>
+          <t>https://www.tiktok.com/@saintmary.sobo</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>salehafoyez</t>
+          <t>ruas_dream</t>
         </is>
       </c>
       <c r="B190" t="inlineStr"/>
@@ -8006,24 +8014,24 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>2026-10-08 19:14:34</t>
+          <t>2026-09-27 11:00:34</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@salehafoyez</t>
+          <t>https://www.tiktok.com/@ruas_dream</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>rtamakter</t>
+          <t>salehafoyez</t>
         </is>
       </c>
       <c r="B191" t="inlineStr"/>
@@ -8040,41 +8048,41 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>2026-10-05 22:45:22</t>
+          <t>2026-10-08 19:14:34</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@rtamakter</t>
+          <t>https://www.tiktok.com/@salehafoyez</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>omo.taiwo11</t>
+          <t>samslittleluxuries</t>
         </is>
       </c>
       <c r="B192" t="inlineStr"/>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>2026-10-11 01:27:22</t>
+          <t>2026-10-11 13:14:02</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -8084,14 +8092,14 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@omo.taiwo11</t>
+          <t>https://www.tiktok.com/@samslittleluxuries</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>oluyewi</t>
+          <t>onos282</t>
         </is>
       </c>
       <c r="B193" t="inlineStr"/>
@@ -8108,31 +8116,31 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-10-03 19:19:51</t>
+          <t>2026-10-04 23:21:40</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oluyewi</t>
+          <t>https://www.tiktok.com/@onos282</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>oluwatoyin0322</t>
+          <t>omo.taiwo11</t>
         </is>
       </c>
       <c r="B194" t="inlineStr"/>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -8142,24 +8150,24 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>2026-09-28 23:38:06</t>
+          <t>2026-10-11 01:27:22</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@oluwatoyin0322</t>
+          <t>https://www.tiktok.com/@omo.taiwo11</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>nonochou12</t>
+          <t>oluyewi</t>
         </is>
       </c>
       <c r="B195" t="inlineStr"/>
@@ -8171,29 +8179,29 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>2026-09-28 00:42:49</t>
+          <t>2026-10-03 19:19:51</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nonochou12</t>
+          <t>https://www.tiktok.com/@oluyewi</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>onos282</t>
+          <t>oluwatoyin0322</t>
         </is>
       </c>
       <c r="B196" t="inlineStr"/>
@@ -8205,22 +8213,22 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>2026-10-04 23:21:40</t>
+          <t>2026-09-28 23:38:06</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@onos282</t>
+          <t>https://www.tiktok.com/@oluwatoyin0322</t>
         </is>
       </c>
     </row>
@@ -8295,41 +8303,41 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>samslittleluxuries</t>
+          <t>riderrrr70</t>
         </is>
       </c>
       <c r="B199" t="inlineStr"/>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
-          <t>[Advent Calendar] 2026</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-10-11 13:14:02</t>
+          <t>2026-09-27 14:15:10</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@samslittleluxuries</t>
+          <t>https://www.tiktok.com/@riderrrr70</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>mary.5884</t>
+          <t>rks_m</t>
         </is>
       </c>
       <c r="B200" t="inlineStr"/>
@@ -8346,7 +8354,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>2026-10-11 12:52:05</t>
+          <t>2026-10-11 19:01:51</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -8356,21 +8364,21 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mary.5884</t>
+          <t>https://www.tiktok.com/@rks_m</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>luulawes2</t>
+          <t>mary.5884</t>
         </is>
       </c>
       <c r="B201" t="inlineStr"/>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
@@ -8380,92 +8388,92 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>2026-10-07 19:43:07</t>
+          <t>2026-10-11 12:52:05</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@luulawes2</t>
+          <t>https://www.tiktok.com/@mary.5884</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>lolaclothier</t>
+          <t>luulawes2</t>
         </is>
       </c>
       <c r="B202" t="inlineStr"/>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>2026-10-01 20:17:12</t>
+          <t>2026-10-07 19:43:07</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@lolaclothier</t>
+          <t>https://www.tiktok.com/@luulawes2</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>london19671962</t>
+          <t>lolaclothier</t>
         </is>
       </c>
       <c r="B203" t="inlineStr"/>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>2026-10-07 20:54:09</t>
+          <t>2026-10-01 20:17:12</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@london19671962</t>
+          <t>https://www.tiktok.com/@lolaclothier</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>laidem4eva</t>
+          <t>london19671962</t>
         </is>
       </c>
       <c r="B204" t="inlineStr"/>
@@ -8482,17 +8490,17 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>2026-10-09 21:38:55</t>
+          <t>2026-10-07 20:54:09</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@laidem4eva</t>
+          <t>https://www.tiktok.com/@london19671962</t>
         </is>
       </c>
     </row>
@@ -8533,14 +8541,14 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>lilliemurrayx</t>
+          <t>laidem4eva</t>
         </is>
       </c>
       <c r="B206" t="inlineStr"/>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E206" t="inlineStr">
@@ -8550,7 +8558,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>2026-10-09 12:08:02</t>
+          <t>2026-10-09 21:38:55</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -8560,21 +8568,21 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@lilliemurrayx</t>
+          <t>https://www.tiktok.com/@laidem4eva</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>linzt78</t>
+          <t>lilliemurrayx</t>
         </is>
       </c>
       <c r="B207" t="inlineStr"/>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
@@ -8584,24 +8592,24 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>2026-10-08 07:33:02</t>
+          <t>2026-10-09 12:08:02</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@linzt78</t>
+          <t>https://www.tiktok.com/@lilliemurrayx</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>mrm.foods.opeyemi</t>
+          <t>linzt78</t>
         </is>
       </c>
       <c r="B208" t="inlineStr"/>
@@ -8613,29 +8621,29 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>2026-10-04 20:07:11</t>
+          <t>2026-10-08 07:33:02</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mrm.foods.opeyemi</t>
+          <t>https://www.tiktok.com/@linzt78</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>mr.liverpool885</t>
+          <t>mrm.foods.opeyemi</t>
         </is>
       </c>
       <c r="B209" t="inlineStr"/>
@@ -8652,7 +8660,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>2026-10-04 09:00:20</t>
+          <t>2026-10-04 20:07:11</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -8662,21 +8670,21 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mr.liverpool885</t>
+          <t>https://www.tiktok.com/@mrm.foods.opeyemi</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>michaela.taylor123</t>
+          <t>mr.liverpool885</t>
         </is>
       </c>
       <c r="B210" t="inlineStr"/>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
@@ -8686,24 +8694,24 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>2026-10-11 13:12:04</t>
+          <t>2026-10-04 09:00:20</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@michaela.taylor123</t>
+          <t>https://www.tiktok.com/@mr.liverpool885</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>michellelake00</t>
+          <t>michaela.taylor123</t>
         </is>
       </c>
       <c r="B211" t="inlineStr"/>
@@ -8715,12 +8723,12 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>2026-10-11 17:47:02</t>
+          <t>2026-10-11 13:12:04</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -8730,31 +8738,31 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@michellelake00</t>
+          <t>https://www.tiktok.com/@michaela.taylor123</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>nataliewestugc</t>
+          <t>michellelake00</t>
         </is>
       </c>
       <c r="B212" t="inlineStr"/>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t>[Advent Calendar] 2026</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>2026-10-11 17:39:02</t>
+          <t>2026-10-11 17:47:02</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -8764,7 +8772,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@nataliewestugc</t>
+          <t>https://www.tiktok.com/@michellelake00</t>
         </is>
       </c>
     </row>
@@ -8805,24 +8813,24 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>natureiskey12</t>
+          <t>nataliewestugc</t>
         </is>
       </c>
       <c r="B214" t="inlineStr"/>
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>2026-10-11 17:49:02</t>
+          <t>2026-10-11 17:39:02</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -8832,21 +8840,21 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@natureiskey12</t>
+          <t>https://www.tiktok.com/@nataliewestugc</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>riderrrr70</t>
+          <t>natureiskey12</t>
         </is>
       </c>
       <c r="B215" t="inlineStr"/>
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
@@ -8856,31 +8864,31 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>2026-09-27 14:15:10</t>
+          <t>2026-10-11 17:49:02</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@riderrrr70</t>
+          <t>https://www.tiktok.com/@natureiskey12</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>secxymum</t>
+          <t>nonochou12</t>
         </is>
       </c>
       <c r="B216" t="inlineStr"/>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E216" t="inlineStr">
@@ -8890,92 +8898,92 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>2026-10-10 15:37:38</t>
+          <t>2026-09-28 00:42:49</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@secxymum</t>
+          <t>https://www.tiktok.com/@nonochou12</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>sarahswhimsyfits</t>
+          <t>shareenyousaf</t>
         </is>
       </c>
       <c r="B217" t="inlineStr"/>
       <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Hibiscus</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>2026-10-01 10:50:06</t>
+          <t>2026-09-29 10:13:11</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sarahswhimsyfits</t>
+          <t>https://www.tiktok.com/@shareenyousaf</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>tinae38</t>
+          <t>secxymum</t>
         </is>
       </c>
       <c r="B218" t="inlineStr"/>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Turmeric Curcumin</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-10-06 12:40:02</t>
+          <t>2026-10-10 15:37:38</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tinae38</t>
+          <t>https://www.tiktok.com/@secxymum</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>theweebelfastman</t>
+          <t>sarahswhimsyfits</t>
         </is>
       </c>
       <c r="B219" t="inlineStr"/>
@@ -8987,12 +8995,12 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>2026-10-01 10:48:02</t>
+          <t>2026-10-01 10:50:06</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -9002,21 +9010,21 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@theweebelfastman</t>
+          <t>https://www.tiktok.com/@sarahswhimsyfits</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>theloyalsoul1</t>
+          <t>theweebelfastman</t>
         </is>
       </c>
       <c r="B220" t="inlineStr"/>
       <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Hibiscus</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
@@ -9026,31 +9034,31 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>2026-09-28 20:53:18</t>
+          <t>2026-10-01 10:48:02</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@theloyalsoul1</t>
+          <t>https://www.tiktok.com/@theweebelfastman</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>shopwithme082</t>
+          <t>theloyalsoul1</t>
         </is>
       </c>
       <c r="B221" t="inlineStr"/>
       <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
@@ -9060,31 +9068,31 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>2026-10-09 12:08:04</t>
+          <t>2026-09-28 20:53:18</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shopwithme082</t>
+          <t>https://www.tiktok.com/@theloyalsoul1</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>shareenyousaf</t>
+          <t>shopwithme082</t>
         </is>
       </c>
       <c r="B222" t="inlineStr"/>
       <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -9094,24 +9102,24 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>2026-09-29 10:13:11</t>
+          <t>2026-10-09 12:08:04</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shareenyousaf</t>
+          <t>https://www.tiktok.com/@shopwithme082</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>stelafinds14</t>
+          <t>sidkam58</t>
         </is>
       </c>
       <c r="B223" t="inlineStr"/>
@@ -9123,29 +9131,29 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>2026-10-11 17:49:02</t>
+          <t>2026-10-01 07:57:16</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@stelafinds14</t>
+          <t>https://www.tiktok.com/@sidkam58</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>sidkam58</t>
+          <t>stelafinds14</t>
         </is>
       </c>
       <c r="B224" t="inlineStr"/>
@@ -9157,36 +9165,36 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>2026-10-01 07:57:16</t>
+          <t>2026-10-11 17:49:02</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sidkam58</t>
+          <t>https://www.tiktok.com/@stelafinds14</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tkmama45</t>
+          <t>tinae38</t>
         </is>
       </c>
       <c r="B225" t="inlineStr"/>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Turmeric Curcumin</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -9196,31 +9204,31 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-10-05 07:34:14</t>
+          <t>2026-10-06 12:40:02</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tkmama45</t>
+          <t>https://www.tiktok.com/@tinae38</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>tiktokshopbestbuys4</t>
+          <t>tkmama45</t>
         </is>
       </c>
       <c r="B226" t="inlineStr"/>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Hibiscus</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E226" t="inlineStr">
@@ -9230,65 +9238,65 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2026-10-08 10:41:47</t>
+          <t>2026-10-05 07:34:14</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tiktokshopbestbuys4</t>
+          <t>https://www.tiktok.com/@tkmama45</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>uniquebolfols</t>
+          <t>tiktokshopbestbuys4</t>
         </is>
       </c>
       <c r="B227" t="inlineStr"/>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Hibiscus</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>2026-10-10 09:01:27</t>
+          <t>2026-10-08 10:41:47</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@uniquebolfols</t>
+          <t>https://www.tiktok.com/@tiktokshopbestbuys4</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>umm_zahra0</t>
+          <t>uniquebolfols</t>
         </is>
       </c>
       <c r="B228" t="inlineStr"/>
       <c r="C228" t="inlineStr"/>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E228" t="inlineStr">
@@ -9298,99 +9306,99 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>2026-10-07 07:43:17</t>
+          <t>2026-10-10 09:01:27</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@umm_zahra0</t>
+          <t>https://www.tiktok.com/@uniquebolfols</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>travelwithme_597</t>
+          <t>umm_zahra0</t>
         </is>
       </c>
       <c r="B229" t="inlineStr"/>
       <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>2026-10-11 13:12:03</t>
+          <t>2026-10-07 07:43:17</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@travelwithme_597</t>
+          <t>https://www.tiktok.com/@umm_zahra0</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>tulai.mans</t>
+          <t>travelwithme_597</t>
         </is>
       </c>
       <c r="B230" t="inlineStr"/>
       <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>2026-10-10 16:03:22</t>
+          <t>2026-10-11 13:12:03</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tulai.mans</t>
+          <t>https://www.tiktok.com/@travelwithme_597</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>triedandtestedbackup</t>
+          <t>tulai.mans</t>
         </is>
       </c>
       <c r="B231" t="inlineStr"/>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -9400,31 +9408,31 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>2026-10-11 17:39:02</t>
+          <t>2026-10-10 16:03:22</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@triedandtestedbackup</t>
+          <t>https://www.tiktok.com/@tulai.mans</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>user8258556352859</t>
+          <t>triedandtestedbackup</t>
         </is>
       </c>
       <c r="B232" t="inlineStr"/>
       <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
@@ -9434,24 +9442,24 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-10-03 10:13:16</t>
+          <t>2026-10-11 17:39:02</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user8258556352859</t>
+          <t>https://www.tiktok.com/@triedandtestedbackup</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>user6931802591156</t>
+          <t>user8258556352859</t>
         </is>
       </c>
       <c r="B233" t="inlineStr"/>
@@ -9468,24 +9476,24 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2026-10-01 16:26:50</t>
+          <t>2026-10-03 10:13:16</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user6931802591156</t>
+          <t>https://www.tiktok.com/@user8258556352859</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>user3998147688485</t>
+          <t>user6931802591156</t>
         </is>
       </c>
       <c r="B234" t="inlineStr"/>
@@ -9502,24 +9510,24 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>2026-09-29 09:40:30</t>
+          <t>2026-10-01 16:26:50</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user3998147688485</t>
+          <t>https://www.tiktok.com/@user6931802591156</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>user35110093</t>
+          <t>user3998147688485</t>
         </is>
       </c>
       <c r="B235" t="inlineStr"/>
@@ -9536,24 +9544,24 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>2026-09-28 20:20:27</t>
+          <t>2026-09-29 09:40:30</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user35110093</t>
+          <t>https://www.tiktok.com/@user3998147688485</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>user3000978251</t>
+          <t>user35110093</t>
         </is>
       </c>
       <c r="B236" t="inlineStr"/>
@@ -9570,41 +9578,41 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>2026-10-08 14:54:13</t>
+          <t>2026-09-28 20:20:27</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user3000978251</t>
+          <t>https://www.tiktok.com/@user35110093</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>user1024226144141</t>
+          <t>user3000978251</t>
         </is>
       </c>
       <c r="B237" t="inlineStr"/>
       <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>2026-10-08 21:41:36</t>
+          <t>2026-10-08 14:54:13</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -9614,31 +9622,31 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user1024226144141</t>
+          <t>https://www.tiktok.com/@user3000978251</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>user93500225626390</t>
+          <t>user1024226144141</t>
         </is>
       </c>
       <c r="B238" t="inlineStr"/>
       <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>2026-10-08 16:06:32</t>
+          <t>2026-10-08 21:41:36</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -9648,14 +9656,14 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user93500225626390</t>
+          <t>https://www.tiktok.com/@user1024226144141</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>user9310370027124</t>
+          <t>user93500225626390</t>
         </is>
       </c>
       <c r="B239" t="inlineStr"/>
@@ -9672,160 +9680,160 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-10-01 19:05:18</t>
+          <t>2026-10-08 16:06:32</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user9310370027124</t>
+          <t>https://www.tiktok.com/@user93500225626390</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>whitneyrianebeautycare</t>
+          <t>user9310370027124</t>
         </is>
       </c>
       <c r="B240" t="inlineStr"/>
       <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>2026-10-11 13:12:03</t>
+          <t>2026-10-01 19:05:18</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@whitneyrianebeautycare</t>
+          <t>https://www.tiktok.com/@user9310370027124</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>waynesear1</t>
+          <t>whitneyrianebeautycare</t>
         </is>
       </c>
       <c r="B241" t="inlineStr"/>
       <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>2026-10-08 17:27:34</t>
+          <t>2026-10-11 13:12:03</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@waynesear1</t>
+          <t>https://www.tiktok.com/@whitneyrianebeautycare</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>waboti</t>
+          <t>waynesear1</t>
         </is>
       </c>
       <c r="B242" t="inlineStr"/>
       <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>2026-10-01 18:00:40</t>
+          <t>2026-10-08 17:27:34</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@waboti</t>
+          <t>https://www.tiktok.com/@waynesear1</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>user99851967341610</t>
+          <t>waboti</t>
         </is>
       </c>
       <c r="B243" t="inlineStr"/>
       <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Green Burner</t>
+          <t>Ashwagandha Coffee</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>2026-09-28 16:59:33</t>
+          <t>2026-10-01 18:00:40</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@user99851967341610</t>
+          <t>https://www.tiktok.com/@waboti</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yeterecipe</t>
+          <t>user99851967341610</t>
         </is>
       </c>
       <c r="B244" t="inlineStr"/>
@@ -9842,24 +9850,24 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>2026-10-02 16:32:43</t>
+          <t>2026-09-28 16:59:33</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@yeterecipe</t>
+          <t>https://www.tiktok.com/@user99851967341610</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>ximenesiane3</t>
+          <t>yeterecipe</t>
         </is>
       </c>
       <c r="B245" t="inlineStr"/>
@@ -9876,31 +9884,31 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>2026-10-07 15:38:53</t>
+          <t>2026-10-02 16:32:43</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ximenesiane3</t>
+          <t>https://www.tiktok.com/@yeterecipe</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>www.tiktokhafsaqueen169</t>
+          <t>ximenesiane3</t>
         </is>
       </c>
       <c r="B246" t="inlineStr"/>
       <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>Green Burner</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
@@ -9910,49 +9918,83 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>2026-09-29 14:46:03</t>
+          <t>2026-10-07 15:38:53</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@www.tiktokhafsaqueen169</t>
+          <t>https://www.tiktok.com/@ximenesiane3</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>zainyzee39</t>
+          <t>www.tiktokhafsaqueen169</t>
         </is>
       </c>
       <c r="B247" t="inlineStr"/>
       <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
+          <t>Ashwagandha Coffee</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Free sample from TikTok Shop (FBT)</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:46:03</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@www.tiktokhafsaqueen169</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>zainyzee39</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr"/>
+      <c r="C248" t="inlineStr"/>
+      <c r="D248" t="inlineStr">
+        <is>
           <t>Green Burner</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>Free sample from seller</t>
-        </is>
-      </c>
-      <c r="F247" t="inlineStr">
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Free sample from seller</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
         <is>
           <t>2026-10-04 10:59:50</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr">
+      <c r="G248" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr">
+      <c r="H248" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@zainyzee39</t>
         </is>

</xml_diff>

<commit_message>
Daily build: data complete through 2026-10-13 (19,131 orders, 13,856 creators); send-level overdue workbook
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -3283,7 +3283,7 @@
         <v>250</v>
       </c>
       <c r="E35" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F35" t="s">
         <v>287</v>
@@ -4652,7 +4652,7 @@
         <v>254</v>
       </c>
       <c r="E88" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F88" t="s">
         <v>284</v>
@@ -6929,7 +6929,7 @@
         <v>250</v>
       </c>
       <c r="E190" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F190" t="s">
         <v>270</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-20 17:40
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Ashwagandha Coffee</t>
+          <t>[Advent Calendar] 2026</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -8919,7 +8919,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Free sample from TikTok Shop (FBT)</t>
+          <t>Free sample from seller</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
@@ -12687,7 +12687,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Free sample from seller</t>
+          <t>Free sample from TikTok Shop (FBT)</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 06:32
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -9487,7 +9487,7 @@
         <v>646</v>
       </c>
       <c r="E158" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F158" t="s">
         <v>772</v>
@@ -9588,7 +9588,7 @@
         <v>641</v>
       </c>
       <c r="D162" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="E162" t="s">
         <v>653</v>
@@ -11561,7 +11561,7 @@
         <v>634</v>
       </c>
       <c r="D238" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="E238" t="s">
         <v>653</v>
@@ -12084,7 +12084,7 @@
         <v>645</v>
       </c>
       <c r="E258" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F258" t="s">
         <v>824</v>
@@ -13072,7 +13072,7 @@
         <v>646</v>
       </c>
       <c r="E296" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F296" t="s">
         <v>848</v>
@@ -13358,7 +13358,7 @@
         <v>646</v>
       </c>
       <c r="E307" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F307" t="s">
         <v>857</v>
@@ -13407,7 +13407,7 @@
         <v>644</v>
       </c>
       <c r="E309" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F309" t="s">
         <v>859</v>
@@ -13927,7 +13927,7 @@
         <v>647</v>
       </c>
       <c r="E329" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F329" t="s">
         <v>868</v>
@@ -15016,7 +15016,7 @@
         <v>647</v>
       </c>
       <c r="E371" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F371" t="s">
         <v>889</v>
@@ -15195,7 +15195,7 @@
         <v>638</v>
       </c>
       <c r="D378" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E378" t="s">
         <v>654</v>
@@ -15221,7 +15221,7 @@
         <v>638</v>
       </c>
       <c r="D379" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="E379" t="s">
         <v>654</v>
@@ -15611,7 +15611,7 @@
         <v>647</v>
       </c>
       <c r="E394" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F394" t="s">
         <v>896</v>
@@ -15946,7 +15946,7 @@
         <v>638</v>
       </c>
       <c r="D407" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="E407" t="s">
         <v>654</v>
@@ -15975,7 +15975,7 @@
         <v>647</v>
       </c>
       <c r="E408" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F408" t="s">
         <v>903</v>
@@ -16738,7 +16738,7 @@
         <v>449</v>
       </c>
       <c r="D443" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="E443" t="s">
         <v>654</v>
@@ -17464,7 +17464,7 @@
         <v>645</v>
       </c>
       <c r="E479" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F479" t="s">
         <v>871</v>
@@ -18882,7 +18882,7 @@
         <v>645</v>
       </c>
       <c r="E549" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F549" t="s">
         <v>832</v>
@@ -19459,7 +19459,7 @@
         <v>584</v>
       </c>
       <c r="D578" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E578" t="s">
         <v>653</v>
@@ -20231,7 +20231,7 @@
         <v>622</v>
       </c>
       <c r="D616" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="E616" t="s">
         <v>653</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-23 06:31
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4347" uniqueCount="1469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4348" uniqueCount="1469">
   <si>
     <t>handle</t>
   </si>
@@ -979,12 +979,12 @@
     <t>fragrance.tok84</t>
   </si>
   <si>
+    <t>annytiktokbuys</t>
+  </si>
+  <si>
     <t>xmxglasgow</t>
   </si>
   <si>
-    <t>annytiktokbuys</t>
-  </si>
-  <si>
     <t>iammemesara1</t>
   </si>
   <si>
@@ -1057,6 +1057,9 @@
     <t>helenjake5</t>
   </si>
   <si>
+    <t>zaman_7024</t>
+  </si>
+  <si>
     <t>lola33684</t>
   </si>
   <si>
@@ -1087,12 +1090,12 @@
     <t>blessedangel404</t>
   </si>
   <si>
+    <t>kariann00</t>
+  </si>
+  <si>
     <t>ewelinawybraniec94</t>
   </si>
   <si>
-    <t>kariann00</t>
-  </si>
-  <si>
     <t>bellasboxesuk</t>
   </si>
   <si>
@@ -1141,12 +1144,12 @@
     <t>bismil_lah77</t>
   </si>
   <si>
+    <t>katiettfinds</t>
+  </si>
+  <si>
     <t>andreirobert50</t>
   </si>
   <si>
-    <t>katiettfinds</t>
-  </si>
-  <si>
     <t>vibe_pozitiv_shop</t>
   </si>
   <si>
@@ -1156,12 +1159,12 @@
     <t>nazmacreates</t>
   </si>
   <si>
+    <t>bookgirlykira27</t>
+  </si>
+  <si>
     <t>ashleighlouisex0</t>
   </si>
   <si>
-    <t>bookgirlykira27</t>
-  </si>
-  <si>
     <t>parisschantelle</t>
   </si>
   <si>
@@ -1198,12 +1201,12 @@
     <t>237nath25</t>
   </si>
   <si>
+    <t>kimlilyandpaws</t>
+  </si>
+  <si>
     <t>gailnorris</t>
   </si>
   <si>
-    <t>kimlilyandpaws</t>
-  </si>
-  <si>
     <t>louisesoutar44</t>
   </si>
   <si>
@@ -1273,12 +1276,12 @@
     <t>angyitseme</t>
   </si>
   <si>
+    <t>joys_journey8</t>
+  </si>
+  <si>
     <t>shelleyzohra10</t>
   </si>
   <si>
-    <t>joys_journey8</t>
-  </si>
-  <si>
     <t>xame_erah4</t>
   </si>
   <si>
@@ -1426,24 +1429,24 @@
     <t>_k_dior</t>
   </si>
   <si>
+    <t>danamason15</t>
+  </si>
+  <si>
     <t>ishratwaheed1</t>
   </si>
   <si>
-    <t>danamason15</t>
-  </si>
-  <si>
     <t>gorgeousgirls6</t>
   </si>
   <si>
     <t>just_advertise</t>
   </si>
   <si>
+    <t>esineade</t>
+  </si>
+  <si>
     <t>clareulettakeeble</t>
   </si>
   <si>
-    <t>esineade</t>
-  </si>
-  <si>
     <t>weemorganwiththebargains</t>
   </si>
   <si>
@@ -1465,12 +1468,12 @@
     <t>moriommodestjourney</t>
   </si>
   <si>
+    <t>nataliewestugc</t>
+  </si>
+  <si>
     <t>anna.pen5</t>
   </si>
   <si>
-    <t>nataliewestugc</t>
-  </si>
-  <si>
     <t>aineyakeel2</t>
   </si>
   <si>
@@ -1498,45 +1501,45 @@
     <t>luxenest20</t>
   </si>
   <si>
+    <t>noob_master69_01</t>
+  </si>
+  <si>
     <t>decentgril11</t>
   </si>
   <si>
-    <t>noob_master69_01</t>
-  </si>
-  <si>
     <t>wanderinglily13</t>
   </si>
   <si>
+    <t>munching_meg</t>
+  </si>
+  <si>
     <t>fissybanky7</t>
   </si>
   <si>
-    <t>munching_meg</t>
+    <t>shecreatesbeauty</t>
   </si>
   <si>
     <t>noor.in.north</t>
   </si>
   <si>
-    <t>shecreatesbeauty</t>
-  </si>
-  <si>
     <t>bellskee42</t>
   </si>
   <si>
     <t>toyosiuk</t>
   </si>
   <si>
+    <t>jodie_bo</t>
+  </si>
+  <si>
     <t>maedaukfinds</t>
   </si>
   <si>
-    <t>jodie_bo</t>
+    <t>maggie_the_magpie1</t>
   </si>
   <si>
     <t>luckyfamily1111</t>
   </si>
   <si>
-    <t>maggie_the_magpie1</t>
-  </si>
-  <si>
     <t>nicnacpaddywack8</t>
   </si>
   <si>
@@ -1573,12 +1576,12 @@
     <t>alannah_leigh</t>
   </si>
   <si>
+    <t>joshuascotthurrel</t>
+  </si>
+  <si>
     <t>maryaybh71p</t>
   </si>
   <si>
-    <t>joshuascotthurrel</t>
-  </si>
-  <si>
     <t>bissmillahshop3</t>
   </si>
   <si>
@@ -1621,15 +1624,12 @@
     <t>rachieha</t>
   </si>
   <si>
+    <t>winniesnwoofs</t>
+  </si>
+  <si>
     <t>psychicintheprovince</t>
   </si>
   <si>
-    <t>winniesnwoofs</t>
-  </si>
-  <si>
-    <t>zaman_7024</t>
-  </si>
-  <si>
     <t>glowandtelljb</t>
   </si>
   <si>
@@ -2458,12 +2458,12 @@
     <t>2026-10-14 13:21:04</t>
   </si>
   <si>
+    <t>2026-10-15 08:18:02</t>
+  </si>
+  <si>
     <t>2026-10-15 13:44:03</t>
   </si>
   <si>
-    <t>2026-10-15 08:18:02</t>
-  </si>
-  <si>
     <t>2026-10-08 11:06:04</t>
   </si>
   <si>
@@ -2593,12 +2593,12 @@
     <t>2026-10-15 08:18:04</t>
   </si>
   <si>
+    <t>2026-10-07 15:21:02</t>
+  </si>
+  <si>
     <t>2026-10-16 20:14:49</t>
   </si>
   <si>
-    <t>2026-10-07 15:21:02</t>
-  </si>
-  <si>
     <t>2026-10-19 10:53:11</t>
   </si>
   <si>
@@ -2686,12 +2686,12 @@
     <t>2026-10-20 14:06:28</t>
   </si>
   <si>
+    <t>2026-10-17 22:55:23</t>
+  </si>
+  <si>
     <t>2026-10-19 14:06:31</t>
   </si>
   <si>
-    <t>2026-10-17 22:55:23</t>
-  </si>
-  <si>
     <t>2026-10-20 13:56:12</t>
   </si>
   <si>
@@ -3706,12 +3706,12 @@
     <t>https://www.tiktok.com/@fragrance.tok84</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@annytiktokbuys</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@xmxglasgow</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@annytiktokbuys</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@iammemesara1</t>
   </si>
   <si>
@@ -3784,6 +3784,9 @@
     <t>https://www.tiktok.com/@helenjake5</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@zaman_7024</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@lola33684</t>
   </si>
   <si>
@@ -3814,12 +3817,12 @@
     <t>https://www.tiktok.com/@blessedangel404</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@kariann00</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@ewelinawybraniec94</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@kariann00</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@bellasboxesuk</t>
   </si>
   <si>
@@ -3868,12 +3871,12 @@
     <t>https://www.tiktok.com/@bismil_lah77</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@katiettfinds</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@andreirobert50</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@katiettfinds</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@vibe_pozitiv_shop</t>
   </si>
   <si>
@@ -3883,12 +3886,12 @@
     <t>https://www.tiktok.com/@nazmacreates</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@bookgirlykira27</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@ashleighlouisex0</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@bookgirlykira27</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@parisschantelle</t>
   </si>
   <si>
@@ -3925,12 +3928,12 @@
     <t>https://www.tiktok.com/@237nath25</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@kimlilyandpaws</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@gailnorris</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@kimlilyandpaws</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@louisesoutar44</t>
   </si>
   <si>
@@ -4000,12 +4003,12 @@
     <t>https://www.tiktok.com/@angyitseme</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@joys_journey8</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@shelleyzohra10</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@joys_journey8</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@xame_erah4</t>
   </si>
   <si>
@@ -4153,24 +4156,24 @@
     <t>https://www.tiktok.com/@_k_dior</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@danamason15</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@ishratwaheed1</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@danamason15</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@gorgeousgirls6</t>
   </si>
   <si>
     <t>https://www.tiktok.com/@just_advertise</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@esineade</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@clareulettakeeble</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@esineade</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@weemorganwiththebargains</t>
   </si>
   <si>
@@ -4192,12 +4195,12 @@
     <t>https://www.tiktok.com/@moriommodestjourney</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@nataliewestugc</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@anna.pen5</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@nataliewestugc</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@aineyakeel2</t>
   </si>
   <si>
@@ -4225,45 +4228,45 @@
     <t>https://www.tiktok.com/@luxenest20</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@noob_master69_01</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@decentgril11</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@noob_master69_01</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@wanderinglily13</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@munching_meg</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@fissybanky7</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@munching_meg</t>
+    <t>https://www.tiktok.com/@shecreatesbeauty</t>
   </si>
   <si>
     <t>https://www.tiktok.com/@noor.in.north</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@shecreatesbeauty</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@bellskee42</t>
   </si>
   <si>
     <t>https://www.tiktok.com/@toyosiuk</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@jodie_bo</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@maedaukfinds</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@jodie_bo</t>
+    <t>https://www.tiktok.com/@maggie_the_magpie1</t>
   </si>
   <si>
     <t>https://www.tiktok.com/@luckyfamily1111</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@maggie_the_magpie1</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@nicnacpaddywack8</t>
   </si>
   <si>
@@ -4300,12 +4303,12 @@
     <t>https://www.tiktok.com/@alannah_leigh</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@joshuascotthurrel</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@maryaybh71p</t>
   </si>
   <si>
-    <t>https://www.tiktok.com/@joshuascotthurrel</t>
-  </si>
-  <si>
     <t>https://www.tiktok.com/@bissmillahshop3</t>
   </si>
   <si>
@@ -4348,13 +4351,10 @@
     <t>https://www.tiktok.com/@rachieha</t>
   </si>
   <si>
+    <t>https://www.tiktok.com/@winniesnwoofs</t>
+  </si>
+  <si>
     <t>https://www.tiktok.com/@psychicintheprovince</t>
-  </si>
-  <si>
-    <t>https://www.tiktok.com/@winniesnwoofs</t>
-  </si>
-  <si>
-    <t>https://www.tiktok.com/@zaman_7024</t>
   </si>
   <si>
     <t>https://www.tiktok.com/@glowandtelljb</t>
@@ -12912,19 +12912,19 @@
         <v>565</v>
       </c>
       <c r="C315" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D315" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E315" t="s">
         <v>591</v>
       </c>
       <c r="F315" t="s">
-        <v>797</v>
+        <v>749</v>
       </c>
       <c r="G315" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="H315" s="2" t="s">
         <v>1230</v>
@@ -12938,19 +12938,19 @@
         <v>565</v>
       </c>
       <c r="C316" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D316" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E316" t="s">
         <v>591</v>
       </c>
       <c r="F316" t="s">
-        <v>749</v>
+        <v>797</v>
       </c>
       <c r="G316" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H316" s="2" t="s">
         <v>1231</v>
@@ -13587,20 +13587,17 @@
       <c r="B341" t="s">
         <v>565</v>
       </c>
-      <c r="C341" t="s">
-        <v>575</v>
-      </c>
       <c r="D341" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E341" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F341" t="s">
-        <v>605</v>
+        <v>799</v>
       </c>
       <c r="G341" t="s">
-        <v>910</v>
+        <v>903</v>
       </c>
       <c r="H341" s="2" t="s">
         <v>1256</v>
@@ -13617,16 +13614,16 @@
         <v>575</v>
       </c>
       <c r="D342" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="E342" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F342" t="s">
-        <v>770</v>
+        <v>605</v>
       </c>
       <c r="G342" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H342" s="2" t="s">
         <v>1257</v>
@@ -13640,16 +13637,16 @@
         <v>565</v>
       </c>
       <c r="C343" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D343" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E343" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F343" t="s">
-        <v>706</v>
+        <v>770</v>
       </c>
       <c r="G343" t="s">
         <v>906</v>
@@ -13666,19 +13663,19 @@
         <v>565</v>
       </c>
       <c r="C344" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="D344" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E344" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F344" t="s">
-        <v>773</v>
+        <v>706</v>
       </c>
       <c r="G344" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="H344" s="2" t="s">
         <v>1259</v>
@@ -13692,16 +13689,16 @@
         <v>565</v>
       </c>
       <c r="C345" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D345" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E345" t="s">
         <v>591</v>
       </c>
       <c r="F345" t="s">
-        <v>811</v>
+        <v>773</v>
       </c>
       <c r="G345" t="s">
         <v>903</v>
@@ -13717,17 +13714,20 @@
       <c r="B346" t="s">
         <v>565</v>
       </c>
+      <c r="C346" t="s">
+        <v>575</v>
+      </c>
       <c r="D346" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E346" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F346" t="s">
-        <v>747</v>
+        <v>811</v>
       </c>
       <c r="G346" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H346" s="2" t="s">
         <v>1261</v>
@@ -13741,16 +13741,16 @@
         <v>565</v>
       </c>
       <c r="D347" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E347" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F347" t="s">
-        <v>614</v>
+        <v>747</v>
       </c>
       <c r="G347" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="H347" s="2" t="s">
         <v>1262</v>
@@ -13763,17 +13763,14 @@
       <c r="B348" t="s">
         <v>565</v>
       </c>
-      <c r="C348" t="s">
-        <v>578</v>
-      </c>
       <c r="D348" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E348" t="s">
         <v>591</v>
       </c>
       <c r="F348" t="s">
-        <v>812</v>
+        <v>614</v>
       </c>
       <c r="G348" t="s">
         <v>903</v>
@@ -13790,19 +13787,19 @@
         <v>565</v>
       </c>
       <c r="C349" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D349" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E349" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F349" t="s">
-        <v>619</v>
+        <v>812</v>
       </c>
       <c r="G349" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="H349" s="2" t="s">
         <v>1264</v>
@@ -13819,16 +13816,16 @@
         <v>575</v>
       </c>
       <c r="D350" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="E350" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F350" t="s">
-        <v>813</v>
+        <v>619</v>
       </c>
       <c r="G350" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
       <c r="H350" s="2" t="s">
         <v>1265</v>
@@ -13842,19 +13839,19 @@
         <v>565</v>
       </c>
       <c r="C351" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D351" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E351" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F351" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="G351" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="H351" s="2" t="s">
         <v>1266</v>
@@ -13877,7 +13874,7 @@
         <v>590</v>
       </c>
       <c r="F352" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="G352" t="s">
         <v>911</v>
@@ -13894,19 +13891,19 @@
         <v>565</v>
       </c>
       <c r="C353" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="D353" t="s">
         <v>583</v>
       </c>
       <c r="E353" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F353" t="s">
-        <v>757</v>
+        <v>815</v>
       </c>
       <c r="G353" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="H353" s="2" t="s">
         <v>1268</v>
@@ -13920,7 +13917,7 @@
         <v>565</v>
       </c>
       <c r="C354" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D354" t="s">
         <v>583</v>
@@ -13929,10 +13926,10 @@
         <v>591</v>
       </c>
       <c r="F354" t="s">
-        <v>816</v>
+        <v>757</v>
       </c>
       <c r="G354" t="s">
-        <v>915</v>
+        <v>908</v>
       </c>
       <c r="H354" s="2" t="s">
         <v>1269</v>
@@ -13946,7 +13943,7 @@
         <v>565</v>
       </c>
       <c r="C355" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D355" t="s">
         <v>583</v>
@@ -13955,10 +13952,10 @@
         <v>591</v>
       </c>
       <c r="F355" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="G355" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="H355" s="2" t="s">
         <v>1270</v>
@@ -13975,16 +13972,16 @@
         <v>578</v>
       </c>
       <c r="D356" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E356" t="s">
         <v>591</v>
       </c>
       <c r="F356" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="G356" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="H356" s="2" t="s">
         <v>1271</v>
@@ -13997,17 +13994,20 @@
       <c r="B357" t="s">
         <v>565</v>
       </c>
+      <c r="C357" t="s">
+        <v>578</v>
+      </c>
       <c r="D357" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E357" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F357" t="s">
-        <v>784</v>
+        <v>818</v>
       </c>
       <c r="G357" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="H357" s="2" t="s">
         <v>1272</v>
@@ -14020,17 +14020,14 @@
       <c r="B358" t="s">
         <v>565</v>
       </c>
-      <c r="C358" t="s">
-        <v>575</v>
-      </c>
       <c r="D358" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E358" t="s">
         <v>590</v>
       </c>
       <c r="F358" t="s">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="G358" t="s">
         <v>906</v>
@@ -14047,19 +14044,19 @@
         <v>565</v>
       </c>
       <c r="C359" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D359" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E359" t="s">
         <v>590</v>
       </c>
       <c r="F359" t="s">
-        <v>808</v>
+        <v>772</v>
       </c>
       <c r="G359" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="H359" s="2" t="s">
         <v>1274</v>
@@ -14073,16 +14070,16 @@
         <v>565</v>
       </c>
       <c r="C360" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D360" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="E360" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F360" t="s">
-        <v>773</v>
+        <v>808</v>
       </c>
       <c r="G360" t="s">
         <v>903</v>
@@ -14099,19 +14096,19 @@
         <v>565</v>
       </c>
       <c r="C361" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D361" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E361" t="s">
         <v>591</v>
       </c>
       <c r="F361" t="s">
-        <v>677</v>
+        <v>773</v>
       </c>
       <c r="G361" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H361" s="2" t="s">
         <v>1276</v>
@@ -14125,19 +14122,19 @@
         <v>565</v>
       </c>
       <c r="C362" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D362" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E362" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F362" t="s">
-        <v>819</v>
+        <v>677</v>
       </c>
       <c r="G362" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="H362" s="2" t="s">
         <v>1277</v>
@@ -14154,16 +14151,16 @@
         <v>575</v>
       </c>
       <c r="D363" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E363" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F363" t="s">
-        <v>730</v>
+        <v>819</v>
       </c>
       <c r="G363" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="H363" s="2" t="s">
         <v>1278</v>
@@ -14186,10 +14183,10 @@
         <v>591</v>
       </c>
       <c r="F364" t="s">
-        <v>820</v>
+        <v>730</v>
       </c>
       <c r="G364" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="H364" s="2" t="s">
         <v>1279</v>
@@ -14212,7 +14209,7 @@
         <v>591</v>
       </c>
       <c r="F365" t="s">
-        <v>799</v>
+        <v>820</v>
       </c>
       <c r="G365" t="s">
         <v>903</v>
@@ -14232,13 +14229,13 @@
         <v>575</v>
       </c>
       <c r="D366" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E366" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F366" t="s">
-        <v>773</v>
+        <v>799</v>
       </c>
       <c r="G366" t="s">
         <v>903</v>
@@ -14254,14 +14251,17 @@
       <c r="B367" t="s">
         <v>565</v>
       </c>
+      <c r="C367" t="s">
+        <v>575</v>
+      </c>
       <c r="D367" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E367" t="s">
         <v>590</v>
       </c>
       <c r="F367" t="s">
-        <v>750</v>
+        <v>773</v>
       </c>
       <c r="G367" t="s">
         <v>903</v>
@@ -14277,20 +14277,17 @@
       <c r="B368" t="s">
         <v>565</v>
       </c>
-      <c r="C368" t="s">
-        <v>578</v>
-      </c>
       <c r="D368" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E368" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F368" t="s">
-        <v>815</v>
+        <v>750</v>
       </c>
       <c r="G368" t="s">
-        <v>911</v>
+        <v>903</v>
       </c>
       <c r="H368" s="2" t="s">
         <v>1283</v>
@@ -14304,19 +14301,19 @@
         <v>565</v>
       </c>
       <c r="C369" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D369" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E369" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F369" t="s">
-        <v>821</v>
+        <v>814</v>
       </c>
       <c r="G369" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="H369" s="2" t="s">
         <v>1284</v>
@@ -14356,16 +14353,16 @@
         <v>565</v>
       </c>
       <c r="C371" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D371" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E371" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F371" t="s">
-        <v>750</v>
+        <v>821</v>
       </c>
       <c r="G371" t="s">
         <v>903</v>
@@ -14382,19 +14379,19 @@
         <v>565</v>
       </c>
       <c r="C372" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D372" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E372" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F372" t="s">
-        <v>687</v>
+        <v>750</v>
       </c>
       <c r="G372" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H372" s="2" t="s">
         <v>1287</v>
@@ -14408,19 +14405,19 @@
         <v>565</v>
       </c>
       <c r="C373" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D373" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E373" t="s">
         <v>590</v>
       </c>
       <c r="F373" t="s">
-        <v>822</v>
+        <v>687</v>
       </c>
       <c r="G373" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H373" s="2" t="s">
         <v>1288</v>
@@ -14434,7 +14431,7 @@
         <v>565</v>
       </c>
       <c r="C374" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D374" t="s">
         <v>583</v>
@@ -14443,10 +14440,10 @@
         <v>590</v>
       </c>
       <c r="F374" t="s">
-        <v>782</v>
+        <v>822</v>
       </c>
       <c r="G374" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="H374" s="2" t="s">
         <v>1289</v>
@@ -14486,7 +14483,7 @@
         <v>565</v>
       </c>
       <c r="C376" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D376" t="s">
         <v>583</v>
@@ -14495,7 +14492,7 @@
         <v>590</v>
       </c>
       <c r="F376" t="s">
-        <v>824</v>
+        <v>782</v>
       </c>
       <c r="G376" t="s">
         <v>903</v>
@@ -14512,19 +14509,19 @@
         <v>565</v>
       </c>
       <c r="C377" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D377" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E377" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F377" t="s">
-        <v>680</v>
+        <v>824</v>
       </c>
       <c r="G377" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H377" s="2" t="s">
         <v>1292</v>
@@ -14538,19 +14535,19 @@
         <v>565</v>
       </c>
       <c r="C378" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D378" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="E378" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F378" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="G378" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H378" s="2" t="s">
         <v>1293</v>
@@ -14564,19 +14561,19 @@
         <v>565</v>
       </c>
       <c r="C379" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D379" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="E379" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F379" t="s">
-        <v>825</v>
+        <v>677</v>
       </c>
       <c r="G379" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H379" s="2" t="s">
         <v>1294</v>
@@ -14590,19 +14587,19 @@
         <v>565</v>
       </c>
       <c r="C380" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D380" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E380" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F380" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G380" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H380" s="2" t="s">
         <v>1295</v>
@@ -14615,17 +14612,20 @@
       <c r="B381" t="s">
         <v>565</v>
       </c>
+      <c r="C381" t="s">
+        <v>575</v>
+      </c>
       <c r="D381" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E381" t="s">
         <v>590</v>
       </c>
       <c r="F381" t="s">
-        <v>749</v>
+        <v>826</v>
       </c>
       <c r="G381" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H381" s="2" t="s">
         <v>1296</v>
@@ -14638,20 +14638,17 @@
       <c r="B382" t="s">
         <v>565</v>
       </c>
-      <c r="C382" t="s">
-        <v>571</v>
-      </c>
       <c r="D382" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E382" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F382" t="s">
-        <v>827</v>
+        <v>749</v>
       </c>
       <c r="G382" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H382" s="2" t="s">
         <v>1297</v>
@@ -14664,17 +14661,20 @@
       <c r="B383" t="s">
         <v>565</v>
       </c>
+      <c r="C383" t="s">
+        <v>571</v>
+      </c>
       <c r="D383" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E383" t="s">
         <v>591</v>
       </c>
       <c r="F383" t="s">
-        <v>750</v>
+        <v>827</v>
       </c>
       <c r="G383" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H383" s="2" t="s">
         <v>1298</v>
@@ -14687,20 +14687,17 @@
       <c r="B384" t="s">
         <v>565</v>
       </c>
-      <c r="C384" t="s">
-        <v>575</v>
-      </c>
       <c r="D384" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E384" t="s">
         <v>591</v>
       </c>
       <c r="F384" t="s">
-        <v>667</v>
+        <v>750</v>
       </c>
       <c r="G384" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H384" s="2" t="s">
         <v>1299</v>
@@ -14717,16 +14714,16 @@
         <v>575</v>
       </c>
       <c r="D385" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E385" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F385" t="s">
-        <v>789</v>
+        <v>667</v>
       </c>
       <c r="G385" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="H385" s="2" t="s">
         <v>1300</v>
@@ -14739,17 +14736,20 @@
       <c r="B386" t="s">
         <v>565</v>
       </c>
+      <c r="C386" t="s">
+        <v>575</v>
+      </c>
       <c r="D386" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="E386" t="s">
         <v>590</v>
       </c>
       <c r="F386" t="s">
-        <v>677</v>
+        <v>789</v>
       </c>
       <c r="G386" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H386" s="2" t="s">
         <v>1301</v>
@@ -14762,20 +14762,17 @@
       <c r="B387" t="s">
         <v>565</v>
       </c>
-      <c r="C387" t="s">
-        <v>572</v>
-      </c>
       <c r="D387" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="E387" t="s">
         <v>590</v>
       </c>
       <c r="F387" t="s">
-        <v>806</v>
+        <v>677</v>
       </c>
       <c r="G387" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="H387" s="2" t="s">
         <v>1302</v>
@@ -14789,19 +14786,19 @@
         <v>565</v>
       </c>
       <c r="C388" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D388" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E388" t="s">
         <v>590</v>
       </c>
       <c r="F388" t="s">
-        <v>757</v>
+        <v>806</v>
       </c>
       <c r="G388" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H388" s="2" t="s">
         <v>1303</v>
@@ -14844,16 +14841,16 @@
         <v>575</v>
       </c>
       <c r="D390" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E390" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F390" t="s">
-        <v>829</v>
+        <v>757</v>
       </c>
       <c r="G390" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="H390" s="2" t="s">
         <v>1305</v>
@@ -14870,16 +14867,16 @@
         <v>575</v>
       </c>
       <c r="D391" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E391" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F391" t="s">
-        <v>701</v>
+        <v>829</v>
       </c>
       <c r="G391" t="s">
-        <v>906</v>
+        <v>913</v>
       </c>
       <c r="H391" s="2" t="s">
         <v>1306</v>
@@ -14892,17 +14889,20 @@
       <c r="B392" t="s">
         <v>565</v>
       </c>
+      <c r="C392" t="s">
+        <v>575</v>
+      </c>
       <c r="D392" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="E392" t="s">
         <v>590</v>
       </c>
       <c r="F392" t="s">
-        <v>830</v>
+        <v>701</v>
       </c>
       <c r="G392" t="s">
-        <v>915</v>
+        <v>906</v>
       </c>
       <c r="H392" s="2" t="s">
         <v>1307</v>
@@ -14915,20 +14915,17 @@
       <c r="B393" t="s">
         <v>565</v>
       </c>
-      <c r="C393" t="s">
-        <v>574</v>
-      </c>
       <c r="D393" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E393" t="s">
         <v>590</v>
       </c>
       <c r="F393" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="G393" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="H393" s="2" t="s">
         <v>1308</v>
@@ -14941,17 +14938,20 @@
       <c r="B394" t="s">
         <v>565</v>
       </c>
+      <c r="C394" t="s">
+        <v>574</v>
+      </c>
       <c r="D394" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E394" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F394" t="s">
-        <v>761</v>
+        <v>831</v>
       </c>
       <c r="G394" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="H394" s="2" t="s">
         <v>1309</v>
@@ -14964,20 +14964,17 @@
       <c r="B395" t="s">
         <v>565</v>
       </c>
-      <c r="C395" t="s">
-        <v>575</v>
-      </c>
       <c r="D395" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E395" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F395" t="s">
-        <v>832</v>
+        <v>761</v>
       </c>
       <c r="G395" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="H395" s="2" t="s">
         <v>1310</v>
@@ -14991,19 +14988,19 @@
         <v>565</v>
       </c>
       <c r="C396" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D396" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="E396" t="s">
         <v>590</v>
       </c>
       <c r="F396" t="s">
-        <v>721</v>
+        <v>832</v>
       </c>
       <c r="G396" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H396" s="2" t="s">
         <v>1311</v>
@@ -15017,19 +15014,19 @@
         <v>565</v>
       </c>
       <c r="C397" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D397" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="E397" t="s">
         <v>590</v>
       </c>
       <c r="F397" t="s">
-        <v>833</v>
+        <v>721</v>
       </c>
       <c r="G397" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="H397" s="2" t="s">
         <v>1312</v>
@@ -15043,19 +15040,19 @@
         <v>565</v>
       </c>
       <c r="C398" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D398" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E398" t="s">
         <v>590</v>
       </c>
       <c r="F398" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="G398" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="H398" s="2" t="s">
         <v>1313</v>
@@ -15066,22 +15063,22 @@
         <v>405</v>
       </c>
       <c r="B399" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C399" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D399" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E399" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F399" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="G399" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="H399" s="2" t="s">
         <v>1314</v>
@@ -15098,16 +15095,16 @@
         <v>578</v>
       </c>
       <c r="D400" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E400" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F400" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="G400" t="s">
-        <v>913</v>
+        <v>907</v>
       </c>
       <c r="H400" s="2" t="s">
         <v>1315</v>
@@ -15121,19 +15118,19 @@
         <v>566</v>
       </c>
       <c r="C401" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D401" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E401" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F401" t="s">
-        <v>605</v>
+        <v>836</v>
       </c>
       <c r="G401" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="H401" s="2" t="s">
         <v>1316</v>
@@ -15146,17 +15143,20 @@
       <c r="B402" t="s">
         <v>566</v>
       </c>
+      <c r="C402" t="s">
+        <v>575</v>
+      </c>
       <c r="D402" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E402" t="s">
         <v>591</v>
       </c>
       <c r="F402" t="s">
-        <v>799</v>
+        <v>605</v>
       </c>
       <c r="G402" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H402" s="2" t="s">
         <v>1317</v>
@@ -15169,9 +15169,6 @@
       <c r="B403" t="s">
         <v>566</v>
       </c>
-      <c r="C403" t="s">
-        <v>575</v>
-      </c>
       <c r="D403" t="s">
         <v>583</v>
       </c>
@@ -15179,10 +15176,10 @@
         <v>591</v>
       </c>
       <c r="F403" t="s">
-        <v>708</v>
+        <v>799</v>
       </c>
       <c r="G403" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H403" s="2" t="s">
         <v>1318</v>
@@ -15205,7 +15202,7 @@
         <v>591</v>
       </c>
       <c r="F404" t="s">
-        <v>652</v>
+        <v>708</v>
       </c>
       <c r="G404" t="s">
         <v>912</v>
@@ -15225,16 +15222,16 @@
         <v>575</v>
       </c>
       <c r="D405" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E405" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F405" t="s">
-        <v>837</v>
+        <v>652</v>
       </c>
       <c r="G405" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="H405" s="2" t="s">
         <v>1320</v>
@@ -15248,19 +15245,19 @@
         <v>566</v>
       </c>
       <c r="C406" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D406" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E406" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F406" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="G406" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="H406" s="2" t="s">
         <v>1321</v>
@@ -15277,16 +15274,16 @@
         <v>572</v>
       </c>
       <c r="D407" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E407" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F407" t="s">
-        <v>747</v>
+        <v>838</v>
       </c>
       <c r="G407" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="H407" s="2" t="s">
         <v>1322</v>
@@ -15300,19 +15297,19 @@
         <v>566</v>
       </c>
       <c r="C408" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D408" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="E408" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F408" t="s">
-        <v>784</v>
+        <v>747</v>
       </c>
       <c r="G408" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="H408" s="2" t="s">
         <v>1323</v>
@@ -15329,16 +15326,16 @@
         <v>575</v>
       </c>
       <c r="D409" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E409" t="s">
         <v>591</v>
       </c>
       <c r="F409" t="s">
-        <v>839</v>
+        <v>784</v>
       </c>
       <c r="G409" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H409" s="2" t="s">
         <v>1324</v>
@@ -15358,13 +15355,13 @@
         <v>583</v>
       </c>
       <c r="E410" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F410" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="G410" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H410" s="2" t="s">
         <v>1325</v>
@@ -15381,16 +15378,16 @@
         <v>575</v>
       </c>
       <c r="D411" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E411" t="s">
         <v>590</v>
       </c>
       <c r="F411" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="G411" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="H411" s="2" t="s">
         <v>1326</v>
@@ -15407,16 +15404,16 @@
         <v>575</v>
       </c>
       <c r="D412" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E412" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F412" t="s">
-        <v>774</v>
+        <v>841</v>
       </c>
       <c r="G412" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="H412" s="2" t="s">
         <v>1327</v>
@@ -15433,16 +15430,16 @@
         <v>575</v>
       </c>
       <c r="D413" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E413" t="s">
         <v>591</v>
       </c>
       <c r="F413" t="s">
-        <v>801</v>
+        <v>774</v>
       </c>
       <c r="G413" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H413" s="2" t="s">
         <v>1328</v>
@@ -15482,19 +15479,19 @@
         <v>566</v>
       </c>
       <c r="C415" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D415" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="E415" t="s">
         <v>591</v>
       </c>
       <c r="F415" t="s">
-        <v>840</v>
+        <v>801</v>
       </c>
       <c r="G415" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="H415" s="2" t="s">
         <v>1330</v>
@@ -15508,19 +15505,19 @@
         <v>566</v>
       </c>
       <c r="C416" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="D416" t="s">
         <v>587</v>
       </c>
       <c r="E416" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F416" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="G416" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="H416" s="2" t="s">
         <v>1331</v>
@@ -15533,17 +15530,20 @@
       <c r="B417" t="s">
         <v>566</v>
       </c>
+      <c r="C417" t="s">
+        <v>572</v>
+      </c>
       <c r="D417" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E417" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F417" t="s">
-        <v>799</v>
+        <v>843</v>
       </c>
       <c r="G417" t="s">
-        <v>903</v>
+        <v>914</v>
       </c>
       <c r="H417" s="2" t="s">
         <v>1332</v>
@@ -15557,16 +15557,16 @@
         <v>566</v>
       </c>
       <c r="D418" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E418" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F418" t="s">
-        <v>687</v>
+        <v>799</v>
       </c>
       <c r="G418" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H418" s="2" t="s">
         <v>1333</v>
@@ -15579,20 +15579,17 @@
       <c r="B419" t="s">
         <v>566</v>
       </c>
-      <c r="C419" t="s">
-        <v>578</v>
-      </c>
       <c r="D419" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E419" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F419" t="s">
-        <v>742</v>
+        <v>687</v>
       </c>
       <c r="G419" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="H419" s="2" t="s">
         <v>1334</v>
@@ -15606,16 +15603,16 @@
         <v>566</v>
       </c>
       <c r="C420" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D420" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E420" t="s">
         <v>591</v>
       </c>
       <c r="F420" t="s">
-        <v>614</v>
+        <v>742</v>
       </c>
       <c r="G420" t="s">
         <v>903</v>
@@ -15632,7 +15629,7 @@
         <v>566</v>
       </c>
       <c r="C421" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D421" t="s">
         <v>583</v>
@@ -15641,10 +15638,10 @@
         <v>591</v>
       </c>
       <c r="F421" t="s">
-        <v>844</v>
+        <v>614</v>
       </c>
       <c r="G421" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H421" s="2" t="s">
         <v>1336</v>
@@ -15658,7 +15655,7 @@
         <v>566</v>
       </c>
       <c r="C422" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D422" t="s">
         <v>583</v>
@@ -15667,10 +15664,10 @@
         <v>591</v>
       </c>
       <c r="F422" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="G422" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="H422" s="2" t="s">
         <v>1337</v>
@@ -15684,19 +15681,19 @@
         <v>566</v>
       </c>
       <c r="C423" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D423" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E423" t="s">
         <v>591</v>
       </c>
       <c r="F423" t="s">
-        <v>832</v>
+        <v>845</v>
       </c>
       <c r="G423" t="s">
-        <v>910</v>
+        <v>903</v>
       </c>
       <c r="H423" s="2" t="s">
         <v>1338</v>
@@ -15719,10 +15716,10 @@
         <v>591</v>
       </c>
       <c r="F424" t="s">
-        <v>715</v>
+        <v>832</v>
       </c>
       <c r="G424" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H424" s="2" t="s">
         <v>1339</v>
@@ -15736,16 +15733,16 @@
         <v>566</v>
       </c>
       <c r="C425" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D425" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E425" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F425" t="s">
-        <v>697</v>
+        <v>715</v>
       </c>
       <c r="G425" t="s">
         <v>906</v>
@@ -15762,7 +15759,7 @@
         <v>566</v>
       </c>
       <c r="C426" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D426" t="s">
         <v>583</v>
@@ -15771,10 +15768,10 @@
         <v>590</v>
       </c>
       <c r="F426" t="s">
-        <v>749</v>
+        <v>697</v>
       </c>
       <c r="G426" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H426" s="2" t="s">
         <v>1341</v>
@@ -15788,19 +15785,19 @@
         <v>566</v>
       </c>
       <c r="C427" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D427" t="s">
         <v>583</v>
       </c>
       <c r="E427" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F427" t="s">
-        <v>605</v>
+        <v>749</v>
       </c>
       <c r="G427" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H427" s="2" t="s">
         <v>1342</v>
@@ -15814,19 +15811,19 @@
         <v>566</v>
       </c>
       <c r="C428" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D428" t="s">
         <v>583</v>
       </c>
       <c r="E428" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F428" t="s">
-        <v>846</v>
+        <v>605</v>
       </c>
       <c r="G428" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="H428" s="2" t="s">
         <v>1343</v>
@@ -15843,16 +15840,16 @@
         <v>575</v>
       </c>
       <c r="D429" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E429" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F429" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="G429" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="H429" s="2" t="s">
         <v>1344</v>
@@ -15866,19 +15863,19 @@
         <v>566</v>
       </c>
       <c r="C430" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D430" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E430" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F430" t="s">
-        <v>757</v>
+        <v>847</v>
       </c>
       <c r="G430" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H430" s="2" t="s">
         <v>1345</v>
@@ -15901,7 +15898,7 @@
         <v>590</v>
       </c>
       <c r="F431" t="s">
-        <v>687</v>
+        <v>757</v>
       </c>
       <c r="G431" t="s">
         <v>908</v>
@@ -15918,19 +15915,19 @@
         <v>566</v>
       </c>
       <c r="C432" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D432" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E432" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F432" t="s">
-        <v>848</v>
+        <v>687</v>
       </c>
       <c r="G432" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="H432" s="2" t="s">
         <v>1347</v>
@@ -15944,19 +15941,19 @@
         <v>566</v>
       </c>
       <c r="C433" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D433" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E433" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F433" t="s">
-        <v>687</v>
+        <v>848</v>
       </c>
       <c r="G433" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H433" s="2" t="s">
         <v>1348</v>
@@ -15973,16 +15970,16 @@
         <v>575</v>
       </c>
       <c r="D434" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E434" t="s">
         <v>590</v>
       </c>
       <c r="F434" t="s">
-        <v>826</v>
+        <v>687</v>
       </c>
       <c r="G434" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="H434" s="2" t="s">
         <v>1349</v>
@@ -15995,17 +15992,20 @@
       <c r="B435" t="s">
         <v>566</v>
       </c>
+      <c r="C435" t="s">
+        <v>575</v>
+      </c>
       <c r="D435" t="s">
         <v>583</v>
       </c>
       <c r="E435" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F435" t="s">
-        <v>784</v>
+        <v>826</v>
       </c>
       <c r="G435" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="H435" s="2" t="s">
         <v>1350</v>
@@ -16018,9 +16018,6 @@
       <c r="B436" t="s">
         <v>566</v>
       </c>
-      <c r="C436" t="s">
-        <v>572</v>
-      </c>
       <c r="D436" t="s">
         <v>583</v>
       </c>
@@ -16028,10 +16025,10 @@
         <v>591</v>
       </c>
       <c r="F436" t="s">
-        <v>815</v>
+        <v>784</v>
       </c>
       <c r="G436" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="H436" s="2" t="s">
         <v>1351</v>
@@ -16045,19 +16042,19 @@
         <v>566</v>
       </c>
       <c r="C437" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D437" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E437" t="s">
         <v>591</v>
       </c>
       <c r="F437" t="s">
-        <v>661</v>
+        <v>814</v>
       </c>
       <c r="G437" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="H437" s="2" t="s">
         <v>1352</v>
@@ -16074,16 +16071,16 @@
         <v>575</v>
       </c>
       <c r="D438" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E438" t="s">
         <v>591</v>
       </c>
       <c r="F438" t="s">
-        <v>763</v>
+        <v>661</v>
       </c>
       <c r="G438" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H438" s="2" t="s">
         <v>1353</v>
@@ -16097,19 +16094,19 @@
         <v>566</v>
       </c>
       <c r="C439" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D439" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E439" t="s">
         <v>591</v>
       </c>
       <c r="F439" t="s">
-        <v>849</v>
+        <v>763</v>
       </c>
       <c r="G439" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="H439" s="2" t="s">
         <v>1354</v>
@@ -16126,16 +16123,16 @@
         <v>572</v>
       </c>
       <c r="D440" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E440" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F440" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G440" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="H440" s="2" t="s">
         <v>1355</v>
@@ -16152,16 +16149,16 @@
         <v>572</v>
       </c>
       <c r="D441" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="E441" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F441" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="G441" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H441" s="2" t="s">
         <v>1356</v>
@@ -16178,16 +16175,16 @@
         <v>572</v>
       </c>
       <c r="D442" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="E442" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F442" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="G442" t="s">
-        <v>910</v>
+        <v>903</v>
       </c>
       <c r="H442" s="2" t="s">
         <v>1357</v>
@@ -16201,19 +16198,19 @@
         <v>566</v>
       </c>
       <c r="C443" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D443" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E443" t="s">
         <v>590</v>
       </c>
       <c r="F443" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="G443" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="H443" s="2" t="s">
         <v>1358</v>
@@ -16230,16 +16227,16 @@
         <v>575</v>
       </c>
       <c r="D444" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E444" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F444" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="G444" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="H444" s="2" t="s">
         <v>1359</v>
@@ -16253,19 +16250,19 @@
         <v>566</v>
       </c>
       <c r="C445" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D445" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E445" t="s">
         <v>591</v>
       </c>
       <c r="F445" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G445" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="H445" s="2" t="s">
         <v>1360</v>
@@ -16279,19 +16276,19 @@
         <v>566</v>
       </c>
       <c r="C446" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D446" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E446" t="s">
         <v>591</v>
       </c>
       <c r="F446" t="s">
-        <v>753</v>
+        <v>855</v>
       </c>
       <c r="G446" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H446" s="2" t="s">
         <v>1361</v>
@@ -16305,16 +16302,16 @@
         <v>566</v>
       </c>
       <c r="C447" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D447" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E447" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F447" t="s">
-        <v>827</v>
+        <v>753</v>
       </c>
       <c r="G447" t="s">
         <v>910</v>
@@ -16331,19 +16328,19 @@
         <v>566</v>
       </c>
       <c r="C448" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D448" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E448" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F448" t="s">
-        <v>856</v>
+        <v>827</v>
       </c>
       <c r="G448" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H448" s="2" t="s">
         <v>1363</v>
@@ -16357,19 +16354,19 @@
         <v>566</v>
       </c>
       <c r="C449" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D449" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E449" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F449" t="s">
-        <v>692</v>
+        <v>856</v>
       </c>
       <c r="G449" t="s">
-        <v>914</v>
+        <v>903</v>
       </c>
       <c r="H449" s="2" t="s">
         <v>1364</v>
@@ -16389,13 +16386,13 @@
         <v>586</v>
       </c>
       <c r="E450" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F450" t="s">
-        <v>605</v>
+        <v>692</v>
       </c>
       <c r="G450" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="H450" s="2" t="s">
         <v>1365</v>
@@ -16412,13 +16409,13 @@
         <v>575</v>
       </c>
       <c r="D451" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E451" t="s">
         <v>591</v>
       </c>
       <c r="F451" t="s">
-        <v>857</v>
+        <v>605</v>
       </c>
       <c r="G451" t="s">
         <v>910</v>
@@ -16434,6 +16431,9 @@
       <c r="B452" t="s">
         <v>566</v>
       </c>
+      <c r="C452" t="s">
+        <v>575</v>
+      </c>
       <c r="D452" t="s">
         <v>583</v>
       </c>
@@ -16441,10 +16441,10 @@
         <v>591</v>
       </c>
       <c r="F452" t="s">
-        <v>614</v>
+        <v>857</v>
       </c>
       <c r="G452" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H452" s="2" t="s">
         <v>1367</v>
@@ -16458,16 +16458,16 @@
         <v>566</v>
       </c>
       <c r="D453" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E453" t="s">
         <v>591</v>
       </c>
       <c r="F453" t="s">
-        <v>753</v>
+        <v>614</v>
       </c>
       <c r="G453" t="s">
-        <v>910</v>
+        <v>903</v>
       </c>
       <c r="H453" s="2" t="s">
         <v>1368</v>
@@ -16480,9 +16480,6 @@
       <c r="B454" t="s">
         <v>566</v>
       </c>
-      <c r="C454" t="s">
-        <v>575</v>
-      </c>
       <c r="D454" t="s">
         <v>586</v>
       </c>
@@ -16490,10 +16487,10 @@
         <v>591</v>
       </c>
       <c r="F454" t="s">
-        <v>782</v>
+        <v>753</v>
       </c>
       <c r="G454" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H454" s="2" t="s">
         <v>1369</v>
@@ -16510,16 +16507,16 @@
         <v>575</v>
       </c>
       <c r="D455" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="E455" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F455" t="s">
-        <v>760</v>
+        <v>782</v>
       </c>
       <c r="G455" t="s">
-        <v>909</v>
+        <v>903</v>
       </c>
       <c r="H455" s="2" t="s">
         <v>1370</v>
@@ -16536,16 +16533,16 @@
         <v>575</v>
       </c>
       <c r="D456" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E456" t="s">
         <v>590</v>
       </c>
       <c r="F456" t="s">
-        <v>750</v>
+        <v>760</v>
       </c>
       <c r="G456" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="H456" s="2" t="s">
         <v>1371</v>
@@ -16559,19 +16556,19 @@
         <v>566</v>
       </c>
       <c r="C457" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D457" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="E457" t="s">
         <v>590</v>
       </c>
       <c r="F457" t="s">
-        <v>858</v>
+        <v>750</v>
       </c>
       <c r="G457" t="s">
-        <v>911</v>
+        <v>903</v>
       </c>
       <c r="H457" s="2" t="s">
         <v>1372</v>
@@ -16585,19 +16582,19 @@
         <v>566</v>
       </c>
       <c r="C458" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D458" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="E458" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F458" t="s">
-        <v>677</v>
+        <v>858</v>
       </c>
       <c r="G458" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="H458" s="2" t="s">
         <v>1373</v>
@@ -16610,17 +16607,20 @@
       <c r="B459" t="s">
         <v>566</v>
       </c>
+      <c r="C459" t="s">
+        <v>572</v>
+      </c>
       <c r="D459" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E459" t="s">
         <v>591</v>
       </c>
       <c r="F459" t="s">
-        <v>761</v>
+        <v>677</v>
       </c>
       <c r="G459" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="H459" s="2" t="s">
         <v>1374</v>
@@ -16633,20 +16633,17 @@
       <c r="B460" t="s">
         <v>566</v>
       </c>
-      <c r="C460" t="s">
-        <v>578</v>
-      </c>
       <c r="D460" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E460" t="s">
         <v>591</v>
       </c>
       <c r="F460" t="s">
-        <v>784</v>
+        <v>761</v>
       </c>
       <c r="G460" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="H460" s="2" t="s">
         <v>1375</v>
@@ -16660,19 +16657,19 @@
         <v>566</v>
       </c>
       <c r="C461" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D461" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E461" t="s">
         <v>591</v>
       </c>
       <c r="F461" t="s">
-        <v>750</v>
+        <v>784</v>
       </c>
       <c r="G461" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="H461" s="2" t="s">
         <v>1376</v>
@@ -16686,19 +16683,19 @@
         <v>566</v>
       </c>
       <c r="C462" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D462" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E462" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F462" t="s">
-        <v>761</v>
+        <v>750</v>
       </c>
       <c r="G462" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H462" s="2" t="s">
         <v>1377</v>
@@ -16712,19 +16709,19 @@
         <v>566</v>
       </c>
       <c r="C463" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D463" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E463" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F463" t="s">
-        <v>833</v>
+        <v>761</v>
       </c>
       <c r="G463" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="H463" s="2" t="s">
         <v>1378</v>
@@ -16738,19 +16735,19 @@
         <v>566</v>
       </c>
       <c r="C464" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D464" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E464" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F464" t="s">
-        <v>859</v>
+        <v>833</v>
       </c>
       <c r="G464" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="H464" s="2" t="s">
         <v>1379</v>
@@ -16773,7 +16770,7 @@
         <v>591</v>
       </c>
       <c r="F465" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="G465" t="s">
         <v>916</v>
@@ -16793,16 +16790,16 @@
         <v>572</v>
       </c>
       <c r="D466" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E466" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F466" t="s">
-        <v>831</v>
+        <v>860</v>
       </c>
       <c r="G466" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H466" s="2" t="s">
         <v>1381</v>
@@ -16816,19 +16813,19 @@
         <v>566</v>
       </c>
       <c r="C467" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D467" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E467" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F467" t="s">
-        <v>861</v>
+        <v>831</v>
       </c>
       <c r="G467" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="H467" s="2" t="s">
         <v>1382</v>
@@ -16845,16 +16842,16 @@
         <v>575</v>
       </c>
       <c r="D468" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="E468" t="s">
         <v>590</v>
       </c>
       <c r="F468" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="G468" t="s">
-        <v>910</v>
+        <v>903</v>
       </c>
       <c r="H468" s="2" t="s">
         <v>1383</v>
@@ -16897,16 +16894,16 @@
         <v>575</v>
       </c>
       <c r="D470" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E470" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F470" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="G470" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="H470" s="2" t="s">
         <v>1385</v>
@@ -16920,19 +16917,19 @@
         <v>566</v>
       </c>
       <c r="C471" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D471" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E471" t="s">
         <v>591</v>
       </c>
       <c r="F471" t="s">
-        <v>666</v>
+        <v>858</v>
       </c>
       <c r="G471" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="H471" s="2" t="s">
         <v>1386</v>
@@ -16946,19 +16943,19 @@
         <v>566</v>
       </c>
       <c r="C472" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D472" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E472" t="s">
         <v>591</v>
       </c>
       <c r="F472" t="s">
-        <v>833</v>
+        <v>666</v>
       </c>
       <c r="G472" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="H472" s="2" t="s">
         <v>1387</v>
@@ -16972,19 +16969,19 @@
         <v>566</v>
       </c>
       <c r="C473" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="D473" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E473" t="s">
         <v>591</v>
       </c>
       <c r="F473" t="s">
-        <v>848</v>
+        <v>833</v>
       </c>
       <c r="G473" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="H473" s="2" t="s">
         <v>1388</v>
@@ -16998,19 +16995,19 @@
         <v>566</v>
       </c>
       <c r="C474" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="D474" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E474" t="s">
         <v>591</v>
       </c>
       <c r="F474" t="s">
-        <v>863</v>
+        <v>848</v>
       </c>
       <c r="G474" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="H474" s="2" t="s">
         <v>1389</v>
@@ -17027,16 +17024,16 @@
         <v>572</v>
       </c>
       <c r="D475" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E475" t="s">
         <v>591</v>
       </c>
       <c r="F475" t="s">
-        <v>826</v>
+        <v>863</v>
       </c>
       <c r="G475" t="s">
-        <v>903</v>
+        <v>913</v>
       </c>
       <c r="H475" s="2" t="s">
         <v>1390</v>
@@ -17050,19 +17047,19 @@
         <v>566</v>
       </c>
       <c r="C476" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D476" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E476" t="s">
         <v>591</v>
       </c>
       <c r="F476" t="s">
-        <v>763</v>
+        <v>826</v>
       </c>
       <c r="G476" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="H476" s="2" t="s">
         <v>1391</v>
@@ -17079,16 +17076,16 @@
         <v>575</v>
       </c>
       <c r="D477" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E477" t="s">
         <v>591</v>
       </c>
       <c r="F477" t="s">
-        <v>864</v>
+        <v>763</v>
       </c>
       <c r="G477" t="s">
-        <v>913</v>
+        <v>906</v>
       </c>
       <c r="H477" s="2" t="s">
         <v>1392</v>
@@ -17127,17 +17124,20 @@
       <c r="B479" t="s">
         <v>566</v>
       </c>
+      <c r="C479" t="s">
+        <v>575</v>
+      </c>
       <c r="D479" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="E479" t="s">
         <v>591</v>
       </c>
       <c r="F479" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="G479" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="H479" s="2" t="s">
         <v>1394</v>
@@ -17150,20 +17150,17 @@
       <c r="B480" t="s">
         <v>566</v>
       </c>
-      <c r="C480" t="s">
-        <v>575</v>
-      </c>
       <c r="D480" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E480" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F480" t="s">
-        <v>762</v>
+        <v>858</v>
       </c>
       <c r="G480" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="H480" s="2" t="s">
         <v>1395</v>
@@ -17177,19 +17174,19 @@
         <v>566</v>
       </c>
       <c r="C481" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D481" t="s">
         <v>585</v>
       </c>
       <c r="E481" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F481" t="s">
-        <v>813</v>
+        <v>762</v>
       </c>
       <c r="G481" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="H481" s="2" t="s">
         <v>1396</v>
@@ -17203,19 +17200,19 @@
         <v>566</v>
       </c>
       <c r="C482" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D482" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E482" t="s">
         <v>591</v>
       </c>
       <c r="F482" t="s">
-        <v>865</v>
+        <v>813</v>
       </c>
       <c r="G482" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="H482" s="2" t="s">
         <v>1397</v>
@@ -17229,19 +17226,19 @@
         <v>566</v>
       </c>
       <c r="C483" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D483" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E483" t="s">
         <v>591</v>
       </c>
       <c r="F483" t="s">
-        <v>850</v>
+        <v>865</v>
       </c>
       <c r="G483" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="H483" s="2" t="s">
         <v>1398</v>
@@ -17258,16 +17255,16 @@
         <v>572</v>
       </c>
       <c r="D484" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E484" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F484" t="s">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="G484" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="H484" s="2" t="s">
         <v>1399</v>
@@ -17281,19 +17278,19 @@
         <v>566</v>
       </c>
       <c r="C485" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D485" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E485" t="s">
         <v>590</v>
       </c>
       <c r="F485" t="s">
-        <v>866</v>
+        <v>837</v>
       </c>
       <c r="G485" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="H485" s="2" t="s">
         <v>1400</v>
@@ -17307,16 +17304,16 @@
         <v>566</v>
       </c>
       <c r="C486" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D486" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="E486" t="s">
         <v>590</v>
       </c>
       <c r="F486" t="s">
-        <v>815</v>
+        <v>866</v>
       </c>
       <c r="G486" t="s">
         <v>911</v>
@@ -17333,19 +17330,19 @@
         <v>566</v>
       </c>
       <c r="C487" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D487" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E487" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F487" t="s">
-        <v>867</v>
+        <v>814</v>
       </c>
       <c r="G487" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="H487" s="2" t="s">
         <v>1402</v>
@@ -17365,13 +17362,13 @@
         <v>583</v>
       </c>
       <c r="E488" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F488" t="s">
-        <v>799</v>
+        <v>867</v>
       </c>
       <c r="G488" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="H488" s="2" t="s">
         <v>1403</v>
@@ -17411,19 +17408,19 @@
         <v>566</v>
       </c>
       <c r="C490" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="D490" t="s">
         <v>583</v>
       </c>
       <c r="E490" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F490" t="s">
-        <v>869</v>
+        <v>799</v>
       </c>
       <c r="G490" t="s">
-        <v>916</v>
+        <v>903</v>
       </c>
       <c r="H490" s="2" t="s">
         <v>1405</v>
@@ -17437,19 +17434,19 @@
         <v>566</v>
       </c>
       <c r="C491" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D491" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E491" t="s">
         <v>591</v>
       </c>
       <c r="F491" t="s">
-        <v>661</v>
+        <v>869</v>
       </c>
       <c r="G491" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
       <c r="H491" s="2" t="s">
         <v>1406</v>
@@ -17492,13 +17489,13 @@
         <v>578</v>
       </c>
       <c r="D493" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="E493" t="s">
         <v>591</v>
       </c>
       <c r="F493" t="s">
-        <v>765</v>
+        <v>661</v>
       </c>
       <c r="G493" t="s">
         <v>910</v>
@@ -17541,19 +17538,19 @@
         <v>566</v>
       </c>
       <c r="C495" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D495" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="E495" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F495" t="s">
-        <v>692</v>
+        <v>765</v>
       </c>
       <c r="G495" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="H495" s="2" t="s">
         <v>1410</v>
@@ -17567,19 +17564,19 @@
         <v>566</v>
       </c>
       <c r="C496" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D496" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="E496" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F496" t="s">
-        <v>872</v>
+        <v>692</v>
       </c>
       <c r="G496" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="H496" s="2" t="s">
         <v>1411</v>
@@ -17593,7 +17590,7 @@
         <v>566</v>
       </c>
       <c r="C497" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D497" t="s">
         <v>586</v>
@@ -17602,10 +17599,10 @@
         <v>591</v>
       </c>
       <c r="F497" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G497" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="H497" s="2" t="s">
         <v>1412</v>
@@ -17648,16 +17645,16 @@
         <v>575</v>
       </c>
       <c r="D499" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="E499" t="s">
         <v>591</v>
       </c>
       <c r="F499" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G499" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="H499" s="2" t="s">
         <v>1414</v>
@@ -17700,16 +17697,16 @@
         <v>575</v>
       </c>
       <c r="D501" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E501" t="s">
         <v>591</v>
       </c>
       <c r="F501" t="s">
-        <v>791</v>
+        <v>874</v>
       </c>
       <c r="G501" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="H501" s="2" t="s">
         <v>1416</v>
@@ -17723,19 +17720,19 @@
         <v>566</v>
       </c>
       <c r="C502" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D502" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E502" t="s">
         <v>591</v>
       </c>
       <c r="F502" t="s">
-        <v>875</v>
+        <v>791</v>
       </c>
       <c r="G502" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="H502" s="2" t="s">
         <v>1417</v>
@@ -17749,16 +17746,16 @@
         <v>566</v>
       </c>
       <c r="C503" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D503" t="s">
         <v>587</v>
       </c>
       <c r="E503" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F503" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="G503" t="s">
         <v>907</v>
@@ -17775,19 +17772,19 @@
         <v>566</v>
       </c>
       <c r="C504" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D504" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="E504" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F504" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="G504" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="H504" s="2" t="s">
         <v>1419</v>
@@ -17798,22 +17795,22 @@
         <v>511</v>
       </c>
       <c r="B505" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C505" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D505" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="E505" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F505" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="G505" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="H505" s="2" t="s">
         <v>1420</v>
@@ -17827,19 +17824,19 @@
         <v>567</v>
       </c>
       <c r="C506" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D506" t="s">
         <v>583</v>
       </c>
       <c r="E506" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F506" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="G506" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H506" s="2" t="s">
         <v>1421</v>
@@ -17853,7 +17850,7 @@
         <v>567</v>
       </c>
       <c r="C507" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D507" t="s">
         <v>583</v>
@@ -17862,7 +17859,7 @@
         <v>591</v>
       </c>
       <c r="F507" t="s">
-        <v>749</v>
+        <v>879</v>
       </c>
       <c r="G507" t="s">
         <v>908</v>
@@ -17882,16 +17879,16 @@
         <v>575</v>
       </c>
       <c r="D508" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E508" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F508" t="s">
-        <v>692</v>
+        <v>749</v>
       </c>
       <c r="G508" t="s">
-        <v>914</v>
+        <v>908</v>
       </c>
       <c r="H508" s="2" t="s">
         <v>1423</v>
@@ -17905,19 +17902,19 @@
         <v>567</v>
       </c>
       <c r="C509" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D509" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="E509" t="s">
         <v>590</v>
       </c>
       <c r="F509" t="s">
-        <v>880</v>
+        <v>692</v>
       </c>
       <c r="G509" t="s">
-        <v>903</v>
+        <v>914</v>
       </c>
       <c r="H509" s="2" t="s">
         <v>1424</v>
@@ -17931,19 +17928,19 @@
         <v>567</v>
       </c>
       <c r="C510" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D510" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E510" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F510" t="s">
-        <v>761</v>
+        <v>880</v>
       </c>
       <c r="G510" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H510" s="2" t="s">
         <v>1425</v>
@@ -17992,7 +17989,7 @@
         <v>591</v>
       </c>
       <c r="F512" t="s">
-        <v>881</v>
+        <v>761</v>
       </c>
       <c r="G512" t="s">
         <v>912</v>
@@ -18009,7 +18006,7 @@
         <v>567</v>
       </c>
       <c r="C513" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D513" t="s">
         <v>583</v>
@@ -18018,7 +18015,7 @@
         <v>591</v>
       </c>
       <c r="F513" t="s">
-        <v>848</v>
+        <v>881</v>
       </c>
       <c r="G513" t="s">
         <v>912</v>
@@ -18061,19 +18058,19 @@
         <v>567</v>
       </c>
       <c r="C515" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D515" t="s">
         <v>583</v>
       </c>
       <c r="E515" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F515" t="s">
-        <v>883</v>
+        <v>848</v>
       </c>
       <c r="G515" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="H515" s="2" t="s">
         <v>1430</v>
@@ -18087,19 +18084,19 @@
         <v>567</v>
       </c>
       <c r="C516" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D516" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E516" t="s">
         <v>590</v>
       </c>
       <c r="F516" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="G516" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="H516" s="2" t="s">
         <v>1431</v>
@@ -18113,19 +18110,19 @@
         <v>567</v>
       </c>
       <c r="C517" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="D517" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E517" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F517" t="s">
-        <v>769</v>
+        <v>884</v>
       </c>
       <c r="G517" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="H517" s="2" t="s">
         <v>1432</v>
@@ -18136,10 +18133,10 @@
         <v>524</v>
       </c>
       <c r="B518" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C518" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="D518" t="s">
         <v>583</v>
@@ -18148,10 +18145,10 @@
         <v>591</v>
       </c>
       <c r="F518" t="s">
-        <v>882</v>
+        <v>769</v>
       </c>
       <c r="G518" t="s">
-        <v>912</v>
+        <v>906</v>
       </c>
       <c r="H518" s="2" t="s">
         <v>1433</v>
@@ -18168,16 +18165,16 @@
         <v>575</v>
       </c>
       <c r="D519" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E519" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F519" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="G519" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="H519" s="2" t="s">
         <v>1434</v>
@@ -18190,17 +18187,20 @@
       <c r="B520" t="s">
         <v>568</v>
       </c>
+      <c r="C520" t="s">
+        <v>575</v>
+      </c>
       <c r="D520" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="E520" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F520" t="s">
-        <v>848</v>
+        <v>885</v>
       </c>
       <c r="G520" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="H520" s="2" t="s">
         <v>1435</v>
@@ -18213,20 +18213,17 @@
       <c r="B521" t="s">
         <v>568</v>
       </c>
-      <c r="C521" t="s">
-        <v>572</v>
-      </c>
       <c r="D521" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="E521" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F521" t="s">
-        <v>886</v>
+        <v>848</v>
       </c>
       <c r="G521" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="H521" s="2" t="s">
         <v>1436</v>
@@ -18240,19 +18237,19 @@
         <v>568</v>
       </c>
       <c r="C522" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D522" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E522" t="s">
         <v>590</v>
       </c>
       <c r="F522" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="G522" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="H522" s="2" t="s">
         <v>1437</v>
@@ -18263,22 +18260,22 @@
         <v>529</v>
       </c>
       <c r="B523" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C523" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D523" t="s">
         <v>583</v>
       </c>
       <c r="E523" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F523" t="s">
-        <v>848</v>
+        <v>887</v>
       </c>
       <c r="G523" t="s">
-        <v>912</v>
+        <v>905</v>
       </c>
       <c r="H523" s="2" t="s">
         <v>1438</v>
@@ -18292,7 +18289,7 @@
         <v>569</v>
       </c>
       <c r="C524" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D524" t="s">
         <v>583</v>
@@ -18318,19 +18315,19 @@
         <v>569</v>
       </c>
       <c r="C525" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="D525" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E525" t="s">
         <v>591</v>
       </c>
       <c r="F525" t="s">
-        <v>888</v>
+        <v>848</v>
       </c>
       <c r="G525" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="H525" s="2" t="s">
         <v>1440</v>
@@ -18344,19 +18341,19 @@
         <v>569</v>
       </c>
       <c r="C526" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D526" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E526" t="s">
         <v>591</v>
       </c>
       <c r="F526" t="s">
-        <v>848</v>
+        <v>888</v>
       </c>
       <c r="G526" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="H526" s="2" t="s">
         <v>1441</v>
@@ -18369,6 +18366,9 @@
       <c r="B527" t="s">
         <v>569</v>
       </c>
+      <c r="C527" t="s">
+        <v>571</v>
+      </c>
       <c r="D527" t="s">
         <v>583</v>
       </c>
@@ -18376,7 +18376,7 @@
         <v>591</v>
       </c>
       <c r="F527" t="s">
-        <v>889</v>
+        <v>848</v>
       </c>
       <c r="G527" t="s">
         <v>912</v>
@@ -18389,17 +18389,20 @@
       <c r="A528" t="s">
         <v>534</v>
       </c>
+      <c r="B528" t="s">
+        <v>569</v>
+      </c>
       <c r="D528" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E528" t="s">
         <v>591</v>
       </c>
       <c r="F528" t="s">
-        <v>770</v>
+        <v>889</v>
       </c>
       <c r="G528" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="H528" s="2" t="s">
         <v>1443</v>
@@ -18409,23 +18412,17 @@
       <c r="A529" t="s">
         <v>535</v>
       </c>
-      <c r="B529" t="s">
-        <v>569</v>
-      </c>
-      <c r="C529" t="s">
-        <v>575</v>
-      </c>
       <c r="D529" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E529" t="s">
         <v>591</v>
       </c>
       <c r="F529" t="s">
-        <v>890</v>
+        <v>770</v>
       </c>
       <c r="G529" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="H529" s="2" t="s">
         <v>1444</v>
@@ -18442,7 +18439,7 @@
         <v>590</v>
       </c>
       <c r="F530" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="G530" t="s">
         <v>905</v>
@@ -18455,6 +18452,12 @@
       <c r="A531" t="s">
         <v>537</v>
       </c>
+      <c r="B531" t="s">
+        <v>569</v>
+      </c>
+      <c r="C531" t="s">
+        <v>575</v>
+      </c>
       <c r="D531" t="s">
         <v>583</v>
       </c>
@@ -18462,7 +18465,7 @@
         <v>591</v>
       </c>
       <c r="F531" t="s">
-        <v>799</v>
+        <v>891</v>
       </c>
       <c r="G531" t="s">
         <v>903</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 07:32
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -6840,7 +6840,7 @@
         <v>617</v>
       </c>
       <c r="E69" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F69" t="s">
         <v>685</v>
@@ -11975,7 +11975,7 @@
         <v>614</v>
       </c>
       <c r="E268" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F268" t="s">
         <v>778</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-27 07:08
</commit_message>
<xml_diff>
--- a/chase_list.xlsx
+++ b/chase_list.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5000" uniqueCount="1696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5002" uniqueCount="1696">
   <si>
     <t>handle</t>
   </si>
@@ -21602,6 +21602,12 @@
     <row r="629" spans="1:8">
       <c r="A629" t="s">
         <v>635</v>
+      </c>
+      <c r="B629" t="s">
+        <v>650</v>
+      </c>
+      <c r="C629" t="s">
+        <v>653</v>
       </c>
       <c r="D629" t="s">
         <v>670</v>

</xml_diff>